<commit_message>
Remove growth size type from accessory categories
</commit_message>
<xml_diff>
--- a/app/download_dir/system_files/шали_по каждому размеру.xlsx
+++ b/app/download_dir/system_files/шали_по каждому размеру.xlsx
@@ -13895,7 +13895,7 @@
   </mergeCells>
   <dataValidations count="11">
     <dataValidation sqref="I7:I1045" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list" errorStyle="stop" operator="between">
-      <formula1>Справочники!$G$2:$G$5</formula1>
+      <formula1>Справочники!$G$2:$G$4</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation sqref="G7:G1045" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="textLength" errorStyle="stop" operator="lessThan">
@@ -14103,7 +14103,7 @@
       </c>
       <c r="G4" s="42" t="inlineStr">
         <is>
-          <t>РОСТ</t>
+          <t>ДЛИНА-ШИРИНА</t>
         </is>
       </c>
       <c r="H4" s="72" t="inlineStr">
@@ -14128,11 +14128,7 @@
           <t>Детск.</t>
         </is>
       </c>
-      <c r="G5" s="42" t="inlineStr">
-        <is>
-          <t>ДЛИНА-ШИРИНА</t>
-        </is>
-      </c>
+      <c r="G5" s="42" t="n"/>
       <c r="H5" s="72" t="inlineStr">
         <is>
           <t>АЗЕРБАЙДЖАН</t>
@@ -16572,7 +16568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E110"/>
+  <dimension ref="B2:E110"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.875" defaultRowHeight="12.75" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19.77" customWidth="1" style="42" min="2" max="2"/>
@@ -16581,7 +16577,6 @@
     <col width="29.63" customWidth="1" style="42" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="12.75" customHeight="1" s="69">
       <c r="B2" s="75" t="inlineStr">
         <is>
@@ -16593,11 +16588,7 @@
           <t>тип размера РОССИЯ</t>
         </is>
       </c>
-      <c r="D2" s="75" t="inlineStr">
-        <is>
-          <t>тип размера РОСТ</t>
-        </is>
-      </c>
+      <c r="D2" s="75" t="n"/>
       <c r="E2" s="75" t="inlineStr">
         <is>
           <t>Тип размера МЕЖДУНАРОДНЫЙ</t>
@@ -16615,11 +16606,7 @@
           <t>18</t>
         </is>
       </c>
-      <c r="D3" s="76" t="inlineStr">
-        <is>
-          <t>50-56</t>
-        </is>
-      </c>
+      <c r="D3" s="76" t="n"/>
       <c r="E3" s="42" t="inlineStr">
         <is>
           <t>2XS</t>
@@ -16637,11 +16624,7 @@
           <t>20</t>
         </is>
       </c>
-      <c r="D4" s="42" t="inlineStr">
-        <is>
-          <t>56-62</t>
-        </is>
-      </c>
+      <c r="D4" s="42" t="n"/>
       <c r="E4" s="76" t="inlineStr">
         <is>
           <t>XS</t>
@@ -16651,7 +16634,7 @@
     <row r="5" ht="12.75" customHeight="1" s="69">
       <c r="B5" s="50" t="inlineStr">
         <is>
-          <t>РОСТ</t>
+          <t>ДЛИНА-ШИРИНА</t>
         </is>
       </c>
       <c r="C5" s="76" t="inlineStr">
@@ -16659,11 +16642,7 @@
           <t>22</t>
         </is>
       </c>
-      <c r="D5" s="76" t="inlineStr">
-        <is>
-          <t xml:space="preserve">62-68 </t>
-        </is>
-      </c>
+      <c r="D5" s="76" t="n"/>
       <c r="E5" s="76" t="inlineStr">
         <is>
           <t>S</t>
@@ -16671,21 +16650,13 @@
       </c>
     </row>
     <row r="6" ht="12.75" customHeight="1" s="69">
-      <c r="B6" s="50" t="inlineStr">
-        <is>
-          <t>ДЛИНА-ШИРИНА</t>
-        </is>
-      </c>
+      <c r="B6" s="50" t="n"/>
       <c r="C6" s="76" t="inlineStr">
         <is>
           <t>24</t>
         </is>
       </c>
-      <c r="D6" s="76" t="inlineStr">
-        <is>
-          <t xml:space="preserve">68-74 </t>
-        </is>
-      </c>
+      <c r="D6" s="76" t="n"/>
       <c r="E6" s="76" t="inlineStr">
         <is>
           <t>M</t>
@@ -16698,11 +16669,7 @@
           <t>26</t>
         </is>
       </c>
-      <c r="D7" s="76" t="inlineStr">
-        <is>
-          <t>74-80</t>
-        </is>
-      </c>
+      <c r="D7" s="76" t="n"/>
       <c r="E7" s="76" t="inlineStr">
         <is>
           <t>L</t>
@@ -16715,11 +16682,7 @@
           <t>28</t>
         </is>
       </c>
-      <c r="D8" s="76" t="inlineStr">
-        <is>
-          <t>80-86</t>
-        </is>
-      </c>
+      <c r="D8" s="76" t="n"/>
       <c r="E8" s="76" t="inlineStr">
         <is>
           <t>XL</t>
@@ -16732,11 +16695,7 @@
           <t>30</t>
         </is>
       </c>
-      <c r="D9" s="42" t="inlineStr">
-        <is>
-          <t>86-92</t>
-        </is>
-      </c>
+      <c r="D9" s="42" t="n"/>
       <c r="E9" s="76" t="inlineStr">
         <is>
           <t>XXL</t>
@@ -16749,11 +16708,7 @@
           <t>32</t>
         </is>
       </c>
-      <c r="D10" s="76" t="inlineStr">
-        <is>
-          <t xml:space="preserve">92-98 </t>
-        </is>
-      </c>
+      <c r="D10" s="76" t="n"/>
       <c r="E10" s="76" t="inlineStr">
         <is>
           <t>XXXL</t>
@@ -16766,11 +16721,7 @@
           <t>34</t>
         </is>
       </c>
-      <c r="D11" s="76" t="inlineStr">
-        <is>
-          <t xml:space="preserve">98-104 </t>
-        </is>
-      </c>
+      <c r="D11" s="76" t="n"/>
       <c r="E11" s="76" t="inlineStr">
         <is>
           <t>4XL</t>
@@ -16783,11 +16734,7 @@
           <t>36</t>
         </is>
       </c>
-      <c r="D12" s="76" t="inlineStr">
-        <is>
-          <t xml:space="preserve">104-110 </t>
-        </is>
-      </c>
+      <c r="D12" s="76" t="n"/>
       <c r="E12" s="76" t="inlineStr">
         <is>
           <t>5XL</t>
@@ -16800,11 +16747,7 @@
           <t>38</t>
         </is>
       </c>
-      <c r="D13" s="76" t="inlineStr">
-        <is>
-          <t xml:space="preserve">110-116 </t>
-        </is>
-      </c>
+      <c r="D13" s="76" t="n"/>
       <c r="E13" s="76" t="inlineStr">
         <is>
           <t>6XL</t>
@@ -16817,11 +16760,7 @@
           <t>40</t>
         </is>
       </c>
-      <c r="D14" s="76" t="inlineStr">
-        <is>
-          <t xml:space="preserve">116-122 </t>
-        </is>
-      </c>
+      <c r="D14" s="76" t="n"/>
       <c r="E14" s="76" t="inlineStr">
         <is>
           <t>7XL</t>
@@ -16834,11 +16773,7 @@
           <t>42</t>
         </is>
       </c>
-      <c r="D15" s="76" t="inlineStr">
-        <is>
-          <t xml:space="preserve">122-128 </t>
-        </is>
-      </c>
+      <c r="D15" s="76" t="n"/>
       <c r="E15" s="76" t="inlineStr">
         <is>
           <t>8XL</t>
@@ -16851,11 +16786,7 @@
           <t>44</t>
         </is>
       </c>
-      <c r="D16" s="76" t="inlineStr">
-        <is>
-          <t xml:space="preserve">128-134 </t>
-        </is>
-      </c>
+      <c r="D16" s="76" t="n"/>
       <c r="E16" s="76" t="inlineStr">
         <is>
           <t>9XL</t>
@@ -16868,11 +16799,7 @@
           <t>46</t>
         </is>
       </c>
-      <c r="D17" s="76" t="inlineStr">
-        <is>
-          <t xml:space="preserve">134-140 </t>
-        </is>
-      </c>
+      <c r="D17" s="76" t="n"/>
       <c r="E17" s="76" t="inlineStr">
         <is>
           <t>10XL</t>
@@ -16885,11 +16812,7 @@
           <t>48</t>
         </is>
       </c>
-      <c r="D18" s="76" t="inlineStr">
-        <is>
-          <t xml:space="preserve">140-146 </t>
-        </is>
-      </c>
+      <c r="D18" s="76" t="n"/>
       <c r="E18" s="76" t="inlineStr">
         <is>
           <t>11XL</t>
@@ -16902,11 +16825,7 @@
           <t>50</t>
         </is>
       </c>
-      <c r="D19" s="76" t="inlineStr">
-        <is>
-          <t>146-152</t>
-        </is>
-      </c>
+      <c r="D19" s="76" t="n"/>
       <c r="E19" s="76" t="inlineStr">
         <is>
           <t>12XL</t>
@@ -16919,11 +16838,7 @@
           <t>52</t>
         </is>
       </c>
-      <c r="D20" s="76" t="inlineStr">
-        <is>
-          <t xml:space="preserve">152-158 </t>
-        </is>
-      </c>
+      <c r="D20" s="76" t="n"/>
       <c r="E20" s="76" t="inlineStr">
         <is>
           <t>13XL</t>
@@ -16936,11 +16851,7 @@
           <t>54</t>
         </is>
       </c>
-      <c r="D21" s="76" t="inlineStr">
-        <is>
-          <t>158-164</t>
-        </is>
-      </c>
+      <c r="D21" s="76" t="n"/>
       <c r="E21" s="76" t="inlineStr">
         <is>
           <t>14XL</t>

</xml_diff>

<commit_message>
Move shawls type aliases to backend
</commit_message>
<xml_diff>
--- a/app/download_dir/system_files/шали_по каждому размеру.xlsx
+++ b/app/download_dir/system_files/шали_по каждому размеру.xlsx
@@ -14784,7 +14784,7 @@
     <row r="44" ht="13.5" customHeight="1" s="69">
       <c r="D44" s="42" t="inlineStr">
         <is>
-          <t>ШАРФ</t>
+          <t>ШАРФ-СНУД</t>
         </is>
       </c>
       <c r="E44" s="42" t="inlineStr">
@@ -16568,7 +16568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="B2:E110"/>
+  <dimension ref="A1:E110"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.875" defaultRowHeight="12.75" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19.77" customWidth="1" style="42" min="2" max="2"/>
@@ -16577,6 +16577,7 @@
     <col width="29.63" customWidth="1" style="42" min="5" max="5"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="12.75" customHeight="1" s="69">
       <c r="B2" s="75" t="inlineStr">
         <is>
@@ -17927,7 +17928,7 @@
     <row r="58" ht="15" customHeight="1" s="69">
       <c r="A58" s="79" t="inlineStr">
         <is>
-          <t>&lt;4000000049&gt; ШАРФ</t>
+          <t>&lt;4000000049&gt; ШАРФ-СНУД</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Port eco fee reporting and weight support
</commit_message>
<xml_diff>
--- a/app/download_dir/system_files/шали_по каждому размеру.xlsx
+++ b/app/download_dir/system_files/шали_по каждому размеру.xlsx
@@ -245,7 +245,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="86">
+  <cellXfs count="87">
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -497,6 +497,9 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -878,19 +881,19 @@
   <dimension ref="A1:AMJ1045"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.43359375" defaultRowHeight="12" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="13.82" customWidth="1" style="42" min="1" max="1"/>
-    <col width="72.34" customWidth="1" style="42" min="2" max="2"/>
+    <col width="13.82" customWidth="1" style="75" min="1" max="1"/>
+    <col width="72.34" customWidth="1" style="75" min="2" max="2"/>
     <col width="47.36" customWidth="1" style="43" min="3" max="3"/>
     <col width="34.53" customWidth="1" style="43" min="4" max="5"/>
     <col width="22.7" customWidth="1" style="43" min="6" max="8"/>
     <col width="24.67" customWidth="1" style="43" min="9" max="9"/>
     <col width="22.7" customWidth="1" style="43" min="10" max="10"/>
     <col width="25.83" customWidth="1" style="43" min="11" max="11"/>
-    <col width="22.7" customWidth="1" style="42" min="12" max="12"/>
+    <col width="22.7" customWidth="1" style="75" min="12" max="12"/>
     <col width="11.35" customWidth="1" style="43" min="14" max="14"/>
-    <col width="17.78" customWidth="1" style="42" min="15" max="15"/>
-    <col width="16" customWidth="1" style="42" min="16" max="16"/>
-    <col width="25.96" customWidth="1" style="42" min="17" max="17"/>
+    <col width="17.78" customWidth="1" style="75" min="15" max="15"/>
+    <col width="16" customWidth="1" style="75" min="16" max="16"/>
+    <col width="25.96" customWidth="1" style="75" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="64.5" customFormat="1" customHeight="1" s="44">
@@ -975,12 +978,12 @@
 ( например 23.10.2023)</t>
         </is>
       </c>
-      <c r="AME1" s="42" t="n"/>
-      <c r="AMF1" s="42" t="n"/>
-      <c r="AMG1" s="42" t="n"/>
-      <c r="AMH1" s="42" t="n"/>
-      <c r="AMI1" s="42" t="n"/>
-      <c r="AMJ1" s="42" t="n"/>
+      <c r="AME1" s="75" t="n"/>
+      <c r="AMF1" s="75" t="n"/>
+      <c r="AMG1" s="75" t="n"/>
+      <c r="AMH1" s="75" t="n"/>
+      <c r="AMI1" s="75" t="n"/>
+      <c r="AMJ1" s="75" t="n"/>
     </row>
     <row r="2" ht="12.75" customFormat="1" customHeight="1" s="44">
       <c r="A2" s="51" t="inlineStr">
@@ -1048,12 +1051,12 @@
       <c r="O2" s="50" t="n"/>
       <c r="P2" s="50" t="n"/>
       <c r="Q2" s="50" t="n"/>
-      <c r="AME2" s="42" t="n"/>
-      <c r="AMF2" s="42" t="n"/>
-      <c r="AMG2" s="42" t="n"/>
-      <c r="AMH2" s="42" t="n"/>
-      <c r="AMI2" s="42" t="n"/>
-      <c r="AMJ2" s="42" t="n"/>
+      <c r="AME2" s="75" t="n"/>
+      <c r="AMF2" s="75" t="n"/>
+      <c r="AMG2" s="75" t="n"/>
+      <c r="AMH2" s="75" t="n"/>
+      <c r="AMI2" s="75" t="n"/>
+      <c r="AMJ2" s="75" t="n"/>
     </row>
     <row r="3" ht="12.75" customFormat="1" customHeight="1" s="44">
       <c r="A3" s="51" t="inlineStr">
@@ -1121,12 +1124,12 @@
       <c r="O3" s="50" t="n"/>
       <c r="P3" s="50" t="n"/>
       <c r="Q3" s="50" t="n"/>
-      <c r="AME3" s="42" t="n"/>
-      <c r="AMF3" s="42" t="n"/>
-      <c r="AMG3" s="42" t="n"/>
-      <c r="AMH3" s="42" t="n"/>
-      <c r="AMI3" s="42" t="n"/>
-      <c r="AMJ3" s="42" t="n"/>
+      <c r="AME3" s="75" t="n"/>
+      <c r="AMF3" s="75" t="n"/>
+      <c r="AMG3" s="75" t="n"/>
+      <c r="AMH3" s="75" t="n"/>
+      <c r="AMI3" s="75" t="n"/>
+      <c r="AMJ3" s="75" t="n"/>
     </row>
     <row r="4" ht="12.75" customFormat="1" customHeight="1" s="44">
       <c r="A4" s="52" t="n"/>
@@ -1190,12 +1193,12 @@
       <c r="O4" s="50" t="n"/>
       <c r="P4" s="50" t="n"/>
       <c r="Q4" s="50" t="n"/>
-      <c r="AME4" s="42" t="n"/>
-      <c r="AMF4" s="42" t="n"/>
-      <c r="AMG4" s="42" t="n"/>
-      <c r="AMH4" s="42" t="n"/>
-      <c r="AMI4" s="42" t="n"/>
-      <c r="AMJ4" s="42" t="n"/>
+      <c r="AME4" s="75" t="n"/>
+      <c r="AMF4" s="75" t="n"/>
+      <c r="AMG4" s="75" t="n"/>
+      <c r="AMH4" s="75" t="n"/>
+      <c r="AMI4" s="75" t="n"/>
+      <c r="AMJ4" s="75" t="n"/>
     </row>
     <row r="5" ht="21.75" customFormat="1" customHeight="1" s="44">
       <c r="A5" s="52" t="n"/>
@@ -1219,12 +1222,12 @@
       <c r="O5" s="54" t="n"/>
       <c r="P5" s="54" t="n"/>
       <c r="Q5" s="54" t="n"/>
-      <c r="AME5" s="42" t="n"/>
-      <c r="AMF5" s="42" t="n"/>
-      <c r="AMG5" s="42" t="n"/>
-      <c r="AMH5" s="42" t="n"/>
-      <c r="AMI5" s="42" t="n"/>
-      <c r="AMJ5" s="42" t="n"/>
+      <c r="AME5" s="75" t="n"/>
+      <c r="AMF5" s="75" t="n"/>
+      <c r="AMG5" s="75" t="n"/>
+      <c r="AMH5" s="75" t="n"/>
+      <c r="AMI5" s="75" t="n"/>
+      <c r="AMJ5" s="75" t="n"/>
     </row>
     <row r="6" ht="202.5" customFormat="1" customHeight="1" s="44">
       <c r="A6" s="55" t="inlineStr">
@@ -1309,12 +1312,12 @@
       </c>
       <c r="P6" s="60" t="n"/>
       <c r="Q6" s="47" t="n"/>
-      <c r="AME6" s="42" t="n"/>
-      <c r="AMF6" s="42" t="n"/>
-      <c r="AMG6" s="42" t="n"/>
-      <c r="AMH6" s="42" t="n"/>
-      <c r="AMI6" s="42" t="n"/>
-      <c r="AMJ6" s="42" t="n"/>
+      <c r="AME6" s="75" t="n"/>
+      <c r="AMF6" s="75" t="n"/>
+      <c r="AMG6" s="75" t="n"/>
+      <c r="AMH6" s="75" t="n"/>
+      <c r="AMI6" s="75" t="n"/>
+      <c r="AMJ6" s="75" t="n"/>
     </row>
     <row r="7" ht="17.25" customFormat="1" customHeight="1" s="61">
       <c r="A7" s="50" t="inlineStr">
@@ -1412,12 +1415,12 @@
       <c r="Z7" s="50" t="n"/>
       <c r="AA7" s="50" t="n"/>
       <c r="AB7" s="50" t="n"/>
-      <c r="AME7" s="42" t="n"/>
-      <c r="AMF7" s="42" t="n"/>
-      <c r="AMG7" s="42" t="n"/>
-      <c r="AMH7" s="42" t="n"/>
-      <c r="AMI7" s="42" t="n"/>
-      <c r="AMJ7" s="42" t="n"/>
+      <c r="AME7" s="75" t="n"/>
+      <c r="AMF7" s="75" t="n"/>
+      <c r="AMG7" s="75" t="n"/>
+      <c r="AMH7" s="75" t="n"/>
+      <c r="AMI7" s="75" t="n"/>
+      <c r="AMJ7" s="75" t="n"/>
     </row>
     <row r="8" ht="17.25" customFormat="1" customHeight="1" s="61">
       <c r="A8" s="50" t="inlineStr">
@@ -1503,12 +1506,12 @@
       <c r="Z8" s="50" t="n"/>
       <c r="AA8" s="50" t="n"/>
       <c r="AB8" s="50" t="n"/>
-      <c r="AME8" s="42" t="n"/>
-      <c r="AMF8" s="42" t="n"/>
-      <c r="AMG8" s="42" t="n"/>
-      <c r="AMH8" s="42" t="n"/>
-      <c r="AMI8" s="42" t="n"/>
-      <c r="AMJ8" s="42" t="n"/>
+      <c r="AME8" s="75" t="n"/>
+      <c r="AMF8" s="75" t="n"/>
+      <c r="AMG8" s="75" t="n"/>
+      <c r="AMH8" s="75" t="n"/>
+      <c r="AMI8" s="75" t="n"/>
+      <c r="AMJ8" s="75" t="n"/>
     </row>
     <row r="9" ht="17.25" customFormat="1" customHeight="1" s="50">
       <c r="B9" s="62">
@@ -1529,12 +1532,12 @@
       <c r="O9" s="68" t="n"/>
       <c r="P9" s="61" t="n"/>
       <c r="Q9" s="61" t="n"/>
-      <c r="AME9" s="42" t="n"/>
-      <c r="AMF9" s="42" t="n"/>
-      <c r="AMG9" s="42" t="n"/>
-      <c r="AMH9" s="42" t="n"/>
-      <c r="AMI9" s="42" t="n"/>
-      <c r="AMJ9" s="42" t="n"/>
+      <c r="AME9" s="75" t="n"/>
+      <c r="AMF9" s="75" t="n"/>
+      <c r="AMG9" s="75" t="n"/>
+      <c r="AMH9" s="75" t="n"/>
+      <c r="AMI9" s="75" t="n"/>
+      <c r="AMJ9" s="75" t="n"/>
     </row>
     <row r="10" ht="17.25" customFormat="1" customHeight="1" s="50">
       <c r="B10" s="62">
@@ -1555,12 +1558,12 @@
       <c r="O10" s="68" t="n"/>
       <c r="P10" s="61" t="n"/>
       <c r="Q10" s="61" t="n"/>
-      <c r="AME10" s="42" t="n"/>
-      <c r="AMF10" s="42" t="n"/>
-      <c r="AMG10" s="42" t="n"/>
-      <c r="AMH10" s="42" t="n"/>
-      <c r="AMI10" s="42" t="n"/>
-      <c r="AMJ10" s="42" t="n"/>
+      <c r="AME10" s="75" t="n"/>
+      <c r="AMF10" s="75" t="n"/>
+      <c r="AMG10" s="75" t="n"/>
+      <c r="AMH10" s="75" t="n"/>
+      <c r="AMI10" s="75" t="n"/>
+      <c r="AMJ10" s="75" t="n"/>
     </row>
     <row r="11" ht="17.25" customFormat="1" customHeight="1" s="50">
       <c r="B11" s="62">
@@ -1581,12 +1584,12 @@
       <c r="O11" s="68" t="n"/>
       <c r="P11" s="61" t="n"/>
       <c r="Q11" s="61" t="n"/>
-      <c r="AME11" s="42" t="n"/>
-      <c r="AMF11" s="42" t="n"/>
-      <c r="AMG11" s="42" t="n"/>
-      <c r="AMH11" s="42" t="n"/>
-      <c r="AMI11" s="42" t="n"/>
-      <c r="AMJ11" s="42" t="n"/>
+      <c r="AME11" s="75" t="n"/>
+      <c r="AMF11" s="75" t="n"/>
+      <c r="AMG11" s="75" t="n"/>
+      <c r="AMH11" s="75" t="n"/>
+      <c r="AMI11" s="75" t="n"/>
+      <c r="AMJ11" s="75" t="n"/>
     </row>
     <row r="12" ht="17.25" customFormat="1" customHeight="1" s="50">
       <c r="B12" s="62">
@@ -1607,12 +1610,12 @@
       <c r="O12" s="68" t="n"/>
       <c r="P12" s="61" t="n"/>
       <c r="Q12" s="61" t="n"/>
-      <c r="AME12" s="42" t="n"/>
-      <c r="AMF12" s="42" t="n"/>
-      <c r="AMG12" s="42" t="n"/>
-      <c r="AMH12" s="42" t="n"/>
-      <c r="AMI12" s="42" t="n"/>
-      <c r="AMJ12" s="42" t="n"/>
+      <c r="AME12" s="75" t="n"/>
+      <c r="AMF12" s="75" t="n"/>
+      <c r="AMG12" s="75" t="n"/>
+      <c r="AMH12" s="75" t="n"/>
+      <c r="AMI12" s="75" t="n"/>
+      <c r="AMJ12" s="75" t="n"/>
     </row>
     <row r="13" ht="17.25" customFormat="1" customHeight="1" s="50">
       <c r="B13" s="62">
@@ -1633,12 +1636,12 @@
       <c r="O13" s="68" t="n"/>
       <c r="P13" s="61" t="n"/>
       <c r="Q13" s="61" t="n"/>
-      <c r="AME13" s="42" t="n"/>
-      <c r="AMF13" s="42" t="n"/>
-      <c r="AMG13" s="42" t="n"/>
-      <c r="AMH13" s="42" t="n"/>
-      <c r="AMI13" s="42" t="n"/>
-      <c r="AMJ13" s="42" t="n"/>
+      <c r="AME13" s="75" t="n"/>
+      <c r="AMF13" s="75" t="n"/>
+      <c r="AMG13" s="75" t="n"/>
+      <c r="AMH13" s="75" t="n"/>
+      <c r="AMI13" s="75" t="n"/>
+      <c r="AMJ13" s="75" t="n"/>
     </row>
     <row r="14" ht="17.25" customFormat="1" customHeight="1" s="50">
       <c r="B14" s="62">
@@ -1659,12 +1662,12 @@
       <c r="O14" s="68" t="n"/>
       <c r="P14" s="61" t="n"/>
       <c r="Q14" s="61" t="n"/>
-      <c r="AME14" s="42" t="n"/>
-      <c r="AMF14" s="42" t="n"/>
-      <c r="AMG14" s="42" t="n"/>
-      <c r="AMH14" s="42" t="n"/>
-      <c r="AMI14" s="42" t="n"/>
-      <c r="AMJ14" s="42" t="n"/>
+      <c r="AME14" s="75" t="n"/>
+      <c r="AMF14" s="75" t="n"/>
+      <c r="AMG14" s="75" t="n"/>
+      <c r="AMH14" s="75" t="n"/>
+      <c r="AMI14" s="75" t="n"/>
+      <c r="AMJ14" s="75" t="n"/>
     </row>
     <row r="15" ht="17.25" customFormat="1" customHeight="1" s="50">
       <c r="B15" s="62">
@@ -1685,12 +1688,12 @@
       <c r="O15" s="68" t="n"/>
       <c r="P15" s="61" t="n"/>
       <c r="Q15" s="61" t="n"/>
-      <c r="AME15" s="42" t="n"/>
-      <c r="AMF15" s="42" t="n"/>
-      <c r="AMG15" s="42" t="n"/>
-      <c r="AMH15" s="42" t="n"/>
-      <c r="AMI15" s="42" t="n"/>
-      <c r="AMJ15" s="42" t="n"/>
+      <c r="AME15" s="75" t="n"/>
+      <c r="AMF15" s="75" t="n"/>
+      <c r="AMG15" s="75" t="n"/>
+      <c r="AMH15" s="75" t="n"/>
+      <c r="AMI15" s="75" t="n"/>
+      <c r="AMJ15" s="75" t="n"/>
     </row>
     <row r="16" ht="17.25" customFormat="1" customHeight="1" s="50">
       <c r="B16" s="62">
@@ -1711,12 +1714,12 @@
       <c r="O16" s="68" t="n"/>
       <c r="P16" s="61" t="n"/>
       <c r="Q16" s="61" t="n"/>
-      <c r="AME16" s="42" t="n"/>
-      <c r="AMF16" s="42" t="n"/>
-      <c r="AMG16" s="42" t="n"/>
-      <c r="AMH16" s="42" t="n"/>
-      <c r="AMI16" s="42" t="n"/>
-      <c r="AMJ16" s="42" t="n"/>
+      <c r="AME16" s="75" t="n"/>
+      <c r="AMF16" s="75" t="n"/>
+      <c r="AMG16" s="75" t="n"/>
+      <c r="AMH16" s="75" t="n"/>
+      <c r="AMI16" s="75" t="n"/>
+      <c r="AMJ16" s="75" t="n"/>
     </row>
     <row r="17" ht="17.25" customFormat="1" customHeight="1" s="50">
       <c r="B17" s="62">
@@ -1737,12 +1740,12 @@
       <c r="O17" s="68" t="n"/>
       <c r="P17" s="61" t="n"/>
       <c r="Q17" s="61" t="n"/>
-      <c r="AME17" s="42" t="n"/>
-      <c r="AMF17" s="42" t="n"/>
-      <c r="AMG17" s="42" t="n"/>
-      <c r="AMH17" s="42" t="n"/>
-      <c r="AMI17" s="42" t="n"/>
-      <c r="AMJ17" s="42" t="n"/>
+      <c r="AME17" s="75" t="n"/>
+      <c r="AMF17" s="75" t="n"/>
+      <c r="AMG17" s="75" t="n"/>
+      <c r="AMH17" s="75" t="n"/>
+      <c r="AMI17" s="75" t="n"/>
+      <c r="AMJ17" s="75" t="n"/>
     </row>
     <row r="18" ht="17.25" customFormat="1" customHeight="1" s="50">
       <c r="B18" s="62">
@@ -1763,12 +1766,12 @@
       <c r="O18" s="68" t="n"/>
       <c r="P18" s="61" t="n"/>
       <c r="Q18" s="61" t="n"/>
-      <c r="AME18" s="42" t="n"/>
-      <c r="AMF18" s="42" t="n"/>
-      <c r="AMG18" s="42" t="n"/>
-      <c r="AMH18" s="42" t="n"/>
-      <c r="AMI18" s="42" t="n"/>
-      <c r="AMJ18" s="42" t="n"/>
+      <c r="AME18" s="75" t="n"/>
+      <c r="AMF18" s="75" t="n"/>
+      <c r="AMG18" s="75" t="n"/>
+      <c r="AMH18" s="75" t="n"/>
+      <c r="AMI18" s="75" t="n"/>
+      <c r="AMJ18" s="75" t="n"/>
     </row>
     <row r="19" ht="17.25" customFormat="1" customHeight="1" s="50">
       <c r="B19" s="62">
@@ -1789,12 +1792,12 @@
       <c r="O19" s="68" t="n"/>
       <c r="P19" s="61" t="n"/>
       <c r="Q19" s="61" t="n"/>
-      <c r="AME19" s="42" t="n"/>
-      <c r="AMF19" s="42" t="n"/>
-      <c r="AMG19" s="42" t="n"/>
-      <c r="AMH19" s="42" t="n"/>
-      <c r="AMI19" s="42" t="n"/>
-      <c r="AMJ19" s="42" t="n"/>
+      <c r="AME19" s="75" t="n"/>
+      <c r="AMF19" s="75" t="n"/>
+      <c r="AMG19" s="75" t="n"/>
+      <c r="AMH19" s="75" t="n"/>
+      <c r="AMI19" s="75" t="n"/>
+      <c r="AMJ19" s="75" t="n"/>
     </row>
     <row r="20" ht="17.25" customFormat="1" customHeight="1" s="50">
       <c r="B20" s="62">
@@ -1815,12 +1818,12 @@
       <c r="O20" s="68" t="n"/>
       <c r="P20" s="61" t="n"/>
       <c r="Q20" s="61" t="n"/>
-      <c r="AME20" s="42" t="n"/>
-      <c r="AMF20" s="42" t="n"/>
-      <c r="AMG20" s="42" t="n"/>
-      <c r="AMH20" s="42" t="n"/>
-      <c r="AMI20" s="42" t="n"/>
-      <c r="AMJ20" s="42" t="n"/>
+      <c r="AME20" s="75" t="n"/>
+      <c r="AMF20" s="75" t="n"/>
+      <c r="AMG20" s="75" t="n"/>
+      <c r="AMH20" s="75" t="n"/>
+      <c r="AMI20" s="75" t="n"/>
+      <c r="AMJ20" s="75" t="n"/>
     </row>
     <row r="21" ht="17.25" customFormat="1" customHeight="1" s="50">
       <c r="B21" s="62">
@@ -1841,12 +1844,12 @@
       <c r="O21" s="68" t="n"/>
       <c r="P21" s="61" t="n"/>
       <c r="Q21" s="61" t="n"/>
-      <c r="AME21" s="42" t="n"/>
-      <c r="AMF21" s="42" t="n"/>
-      <c r="AMG21" s="42" t="n"/>
-      <c r="AMH21" s="42" t="n"/>
-      <c r="AMI21" s="42" t="n"/>
-      <c r="AMJ21" s="42" t="n"/>
+      <c r="AME21" s="75" t="n"/>
+      <c r="AMF21" s="75" t="n"/>
+      <c r="AMG21" s="75" t="n"/>
+      <c r="AMH21" s="75" t="n"/>
+      <c r="AMI21" s="75" t="n"/>
+      <c r="AMJ21" s="75" t="n"/>
     </row>
     <row r="22" ht="17.25" customFormat="1" customHeight="1" s="50">
       <c r="B22" s="62">
@@ -1867,12 +1870,12 @@
       <c r="O22" s="68" t="n"/>
       <c r="P22" s="61" t="n"/>
       <c r="Q22" s="61" t="n"/>
-      <c r="AME22" s="42" t="n"/>
-      <c r="AMF22" s="42" t="n"/>
-      <c r="AMG22" s="42" t="n"/>
-      <c r="AMH22" s="42" t="n"/>
-      <c r="AMI22" s="42" t="n"/>
-      <c r="AMJ22" s="42" t="n"/>
+      <c r="AME22" s="75" t="n"/>
+      <c r="AMF22" s="75" t="n"/>
+      <c r="AMG22" s="75" t="n"/>
+      <c r="AMH22" s="75" t="n"/>
+      <c r="AMI22" s="75" t="n"/>
+      <c r="AMJ22" s="75" t="n"/>
     </row>
     <row r="23" ht="17.25" customFormat="1" customHeight="1" s="50">
       <c r="B23" s="62">
@@ -1893,12 +1896,12 @@
       <c r="O23" s="68" t="n"/>
       <c r="P23" s="61" t="n"/>
       <c r="Q23" s="61" t="n"/>
-      <c r="AME23" s="42" t="n"/>
-      <c r="AMF23" s="42" t="n"/>
-      <c r="AMG23" s="42" t="n"/>
-      <c r="AMH23" s="42" t="n"/>
-      <c r="AMI23" s="42" t="n"/>
-      <c r="AMJ23" s="42" t="n"/>
+      <c r="AME23" s="75" t="n"/>
+      <c r="AMF23" s="75" t="n"/>
+      <c r="AMG23" s="75" t="n"/>
+      <c r="AMH23" s="75" t="n"/>
+      <c r="AMI23" s="75" t="n"/>
+      <c r="AMJ23" s="75" t="n"/>
     </row>
     <row r="24" ht="17.25" customFormat="1" customHeight="1" s="50">
       <c r="B24" s="62">
@@ -1919,12 +1922,12 @@
       <c r="O24" s="68" t="n"/>
       <c r="P24" s="61" t="n"/>
       <c r="Q24" s="61" t="n"/>
-      <c r="AME24" s="42" t="n"/>
-      <c r="AMF24" s="42" t="n"/>
-      <c r="AMG24" s="42" t="n"/>
-      <c r="AMH24" s="42" t="n"/>
-      <c r="AMI24" s="42" t="n"/>
-      <c r="AMJ24" s="42" t="n"/>
+      <c r="AME24" s="75" t="n"/>
+      <c r="AMF24" s="75" t="n"/>
+      <c r="AMG24" s="75" t="n"/>
+      <c r="AMH24" s="75" t="n"/>
+      <c r="AMI24" s="75" t="n"/>
+      <c r="AMJ24" s="75" t="n"/>
     </row>
     <row r="25" ht="17.25" customFormat="1" customHeight="1" s="50">
       <c r="B25" s="62">
@@ -1945,12 +1948,12 @@
       <c r="O25" s="68" t="n"/>
       <c r="P25" s="61" t="n"/>
       <c r="Q25" s="61" t="n"/>
-      <c r="AME25" s="42" t="n"/>
-      <c r="AMF25" s="42" t="n"/>
-      <c r="AMG25" s="42" t="n"/>
-      <c r="AMH25" s="42" t="n"/>
-      <c r="AMI25" s="42" t="n"/>
-      <c r="AMJ25" s="42" t="n"/>
+      <c r="AME25" s="75" t="n"/>
+      <c r="AMF25" s="75" t="n"/>
+      <c r="AMG25" s="75" t="n"/>
+      <c r="AMH25" s="75" t="n"/>
+      <c r="AMI25" s="75" t="n"/>
+      <c r="AMJ25" s="75" t="n"/>
     </row>
     <row r="26" ht="17.25" customFormat="1" customHeight="1" s="50">
       <c r="B26" s="62">
@@ -1971,12 +1974,12 @@
       <c r="O26" s="68" t="n"/>
       <c r="P26" s="61" t="n"/>
       <c r="Q26" s="61" t="n"/>
-      <c r="AME26" s="42" t="n"/>
-      <c r="AMF26" s="42" t="n"/>
-      <c r="AMG26" s="42" t="n"/>
-      <c r="AMH26" s="42" t="n"/>
-      <c r="AMI26" s="42" t="n"/>
-      <c r="AMJ26" s="42" t="n"/>
+      <c r="AME26" s="75" t="n"/>
+      <c r="AMF26" s="75" t="n"/>
+      <c r="AMG26" s="75" t="n"/>
+      <c r="AMH26" s="75" t="n"/>
+      <c r="AMI26" s="75" t="n"/>
+      <c r="AMJ26" s="75" t="n"/>
     </row>
     <row r="27" ht="17.25" customFormat="1" customHeight="1" s="50">
       <c r="B27" s="62">
@@ -1997,12 +2000,12 @@
       <c r="O27" s="68" t="n"/>
       <c r="P27" s="61" t="n"/>
       <c r="Q27" s="61" t="n"/>
-      <c r="AME27" s="42" t="n"/>
-      <c r="AMF27" s="42" t="n"/>
-      <c r="AMG27" s="42" t="n"/>
-      <c r="AMH27" s="42" t="n"/>
-      <c r="AMI27" s="42" t="n"/>
-      <c r="AMJ27" s="42" t="n"/>
+      <c r="AME27" s="75" t="n"/>
+      <c r="AMF27" s="75" t="n"/>
+      <c r="AMG27" s="75" t="n"/>
+      <c r="AMH27" s="75" t="n"/>
+      <c r="AMI27" s="75" t="n"/>
+      <c r="AMJ27" s="75" t="n"/>
     </row>
     <row r="28" ht="17.25" customFormat="1" customHeight="1" s="50">
       <c r="B28" s="62">
@@ -2023,12 +2026,12 @@
       <c r="O28" s="68" t="n"/>
       <c r="P28" s="61" t="n"/>
       <c r="Q28" s="61" t="n"/>
-      <c r="AME28" s="42" t="n"/>
-      <c r="AMF28" s="42" t="n"/>
-      <c r="AMG28" s="42" t="n"/>
-      <c r="AMH28" s="42" t="n"/>
-      <c r="AMI28" s="42" t="n"/>
-      <c r="AMJ28" s="42" t="n"/>
+      <c r="AME28" s="75" t="n"/>
+      <c r="AMF28" s="75" t="n"/>
+      <c r="AMG28" s="75" t="n"/>
+      <c r="AMH28" s="75" t="n"/>
+      <c r="AMI28" s="75" t="n"/>
+      <c r="AMJ28" s="75" t="n"/>
     </row>
     <row r="29" ht="17.25" customFormat="1" customHeight="1" s="50">
       <c r="B29" s="62">
@@ -2049,12 +2052,12 @@
       <c r="O29" s="68" t="n"/>
       <c r="P29" s="61" t="n"/>
       <c r="Q29" s="61" t="n"/>
-      <c r="AME29" s="42" t="n"/>
-      <c r="AMF29" s="42" t="n"/>
-      <c r="AMG29" s="42" t="n"/>
-      <c r="AMH29" s="42" t="n"/>
-      <c r="AMI29" s="42" t="n"/>
-      <c r="AMJ29" s="42" t="n"/>
+      <c r="AME29" s="75" t="n"/>
+      <c r="AMF29" s="75" t="n"/>
+      <c r="AMG29" s="75" t="n"/>
+      <c r="AMH29" s="75" t="n"/>
+      <c r="AMI29" s="75" t="n"/>
+      <c r="AMJ29" s="75" t="n"/>
     </row>
     <row r="30" ht="17.25" customFormat="1" customHeight="1" s="50">
       <c r="B30" s="62">
@@ -2075,12 +2078,12 @@
       <c r="O30" s="68" t="n"/>
       <c r="P30" s="61" t="n"/>
       <c r="Q30" s="61" t="n"/>
-      <c r="AME30" s="42" t="n"/>
-      <c r="AMF30" s="42" t="n"/>
-      <c r="AMG30" s="42" t="n"/>
-      <c r="AMH30" s="42" t="n"/>
-      <c r="AMI30" s="42" t="n"/>
-      <c r="AMJ30" s="42" t="n"/>
+      <c r="AME30" s="75" t="n"/>
+      <c r="AMF30" s="75" t="n"/>
+      <c r="AMG30" s="75" t="n"/>
+      <c r="AMH30" s="75" t="n"/>
+      <c r="AMI30" s="75" t="n"/>
+      <c r="AMJ30" s="75" t="n"/>
     </row>
     <row r="31" ht="17.25" customFormat="1" customHeight="1" s="50">
       <c r="B31" s="62">
@@ -2101,12 +2104,12 @@
       <c r="O31" s="68" t="n"/>
       <c r="P31" s="61" t="n"/>
       <c r="Q31" s="61" t="n"/>
-      <c r="AME31" s="42" t="n"/>
-      <c r="AMF31" s="42" t="n"/>
-      <c r="AMG31" s="42" t="n"/>
-      <c r="AMH31" s="42" t="n"/>
-      <c r="AMI31" s="42" t="n"/>
-      <c r="AMJ31" s="42" t="n"/>
+      <c r="AME31" s="75" t="n"/>
+      <c r="AMF31" s="75" t="n"/>
+      <c r="AMG31" s="75" t="n"/>
+      <c r="AMH31" s="75" t="n"/>
+      <c r="AMI31" s="75" t="n"/>
+      <c r="AMJ31" s="75" t="n"/>
     </row>
     <row r="32" ht="17.25" customFormat="1" customHeight="1" s="50">
       <c r="B32" s="62">
@@ -2127,12 +2130,12 @@
       <c r="O32" s="68" t="n"/>
       <c r="P32" s="61" t="n"/>
       <c r="Q32" s="61" t="n"/>
-      <c r="AME32" s="42" t="n"/>
-      <c r="AMF32" s="42" t="n"/>
-      <c r="AMG32" s="42" t="n"/>
-      <c r="AMH32" s="42" t="n"/>
-      <c r="AMI32" s="42" t="n"/>
-      <c r="AMJ32" s="42" t="n"/>
+      <c r="AME32" s="75" t="n"/>
+      <c r="AMF32" s="75" t="n"/>
+      <c r="AMG32" s="75" t="n"/>
+      <c r="AMH32" s="75" t="n"/>
+      <c r="AMI32" s="75" t="n"/>
+      <c r="AMJ32" s="75" t="n"/>
     </row>
     <row r="33" ht="17.25" customFormat="1" customHeight="1" s="50">
       <c r="B33" s="62">
@@ -2153,12 +2156,12 @@
       <c r="O33" s="68" t="n"/>
       <c r="P33" s="61" t="n"/>
       <c r="Q33" s="61" t="n"/>
-      <c r="AME33" s="42" t="n"/>
-      <c r="AMF33" s="42" t="n"/>
-      <c r="AMG33" s="42" t="n"/>
-      <c r="AMH33" s="42" t="n"/>
-      <c r="AMI33" s="42" t="n"/>
-      <c r="AMJ33" s="42" t="n"/>
+      <c r="AME33" s="75" t="n"/>
+      <c r="AMF33" s="75" t="n"/>
+      <c r="AMG33" s="75" t="n"/>
+      <c r="AMH33" s="75" t="n"/>
+      <c r="AMI33" s="75" t="n"/>
+      <c r="AMJ33" s="75" t="n"/>
     </row>
     <row r="34" ht="17.25" customFormat="1" customHeight="1" s="50">
       <c r="B34" s="62">
@@ -2179,12 +2182,12 @@
       <c r="O34" s="68" t="n"/>
       <c r="P34" s="61" t="n"/>
       <c r="Q34" s="61" t="n"/>
-      <c r="AME34" s="42" t="n"/>
-      <c r="AMF34" s="42" t="n"/>
-      <c r="AMG34" s="42" t="n"/>
-      <c r="AMH34" s="42" t="n"/>
-      <c r="AMI34" s="42" t="n"/>
-      <c r="AMJ34" s="42" t="n"/>
+      <c r="AME34" s="75" t="n"/>
+      <c r="AMF34" s="75" t="n"/>
+      <c r="AMG34" s="75" t="n"/>
+      <c r="AMH34" s="75" t="n"/>
+      <c r="AMI34" s="75" t="n"/>
+      <c r="AMJ34" s="75" t="n"/>
     </row>
     <row r="35" ht="17.25" customFormat="1" customHeight="1" s="50">
       <c r="B35" s="62">
@@ -2205,12 +2208,12 @@
       <c r="O35" s="68" t="n"/>
       <c r="P35" s="61" t="n"/>
       <c r="Q35" s="61" t="n"/>
-      <c r="AME35" s="42" t="n"/>
-      <c r="AMF35" s="42" t="n"/>
-      <c r="AMG35" s="42" t="n"/>
-      <c r="AMH35" s="42" t="n"/>
-      <c r="AMI35" s="42" t="n"/>
-      <c r="AMJ35" s="42" t="n"/>
+      <c r="AME35" s="75" t="n"/>
+      <c r="AMF35" s="75" t="n"/>
+      <c r="AMG35" s="75" t="n"/>
+      <c r="AMH35" s="75" t="n"/>
+      <c r="AMI35" s="75" t="n"/>
+      <c r="AMJ35" s="75" t="n"/>
     </row>
     <row r="36" ht="17.25" customFormat="1" customHeight="1" s="50">
       <c r="B36" s="62">
@@ -2231,12 +2234,12 @@
       <c r="O36" s="68" t="n"/>
       <c r="P36" s="61" t="n"/>
       <c r="Q36" s="61" t="n"/>
-      <c r="AME36" s="42" t="n"/>
-      <c r="AMF36" s="42" t="n"/>
-      <c r="AMG36" s="42" t="n"/>
-      <c r="AMH36" s="42" t="n"/>
-      <c r="AMI36" s="42" t="n"/>
-      <c r="AMJ36" s="42" t="n"/>
+      <c r="AME36" s="75" t="n"/>
+      <c r="AMF36" s="75" t="n"/>
+      <c r="AMG36" s="75" t="n"/>
+      <c r="AMH36" s="75" t="n"/>
+      <c r="AMI36" s="75" t="n"/>
+      <c r="AMJ36" s="75" t="n"/>
     </row>
     <row r="37" ht="17.25" customFormat="1" customHeight="1" s="50">
       <c r="B37" s="62">
@@ -2257,12 +2260,12 @@
       <c r="O37" s="68" t="n"/>
       <c r="P37" s="61" t="n"/>
       <c r="Q37" s="61" t="n"/>
-      <c r="AME37" s="42" t="n"/>
-      <c r="AMF37" s="42" t="n"/>
-      <c r="AMG37" s="42" t="n"/>
-      <c r="AMH37" s="42" t="n"/>
-      <c r="AMI37" s="42" t="n"/>
-      <c r="AMJ37" s="42" t="n"/>
+      <c r="AME37" s="75" t="n"/>
+      <c r="AMF37" s="75" t="n"/>
+      <c r="AMG37" s="75" t="n"/>
+      <c r="AMH37" s="75" t="n"/>
+      <c r="AMI37" s="75" t="n"/>
+      <c r="AMJ37" s="75" t="n"/>
     </row>
     <row r="38" ht="17.25" customFormat="1" customHeight="1" s="50">
       <c r="B38" s="62">
@@ -2283,12 +2286,12 @@
       <c r="O38" s="68" t="n"/>
       <c r="P38" s="61" t="n"/>
       <c r="Q38" s="61" t="n"/>
-      <c r="AME38" s="42" t="n"/>
-      <c r="AMF38" s="42" t="n"/>
-      <c r="AMG38" s="42" t="n"/>
-      <c r="AMH38" s="42" t="n"/>
-      <c r="AMI38" s="42" t="n"/>
-      <c r="AMJ38" s="42" t="n"/>
+      <c r="AME38" s="75" t="n"/>
+      <c r="AMF38" s="75" t="n"/>
+      <c r="AMG38" s="75" t="n"/>
+      <c r="AMH38" s="75" t="n"/>
+      <c r="AMI38" s="75" t="n"/>
+      <c r="AMJ38" s="75" t="n"/>
     </row>
     <row r="39" ht="17.25" customFormat="1" customHeight="1" s="50">
       <c r="B39" s="62">
@@ -2309,12 +2312,12 @@
       <c r="O39" s="68" t="n"/>
       <c r="P39" s="61" t="n"/>
       <c r="Q39" s="61" t="n"/>
-      <c r="AME39" s="42" t="n"/>
-      <c r="AMF39" s="42" t="n"/>
-      <c r="AMG39" s="42" t="n"/>
-      <c r="AMH39" s="42" t="n"/>
-      <c r="AMI39" s="42" t="n"/>
-      <c r="AMJ39" s="42" t="n"/>
+      <c r="AME39" s="75" t="n"/>
+      <c r="AMF39" s="75" t="n"/>
+      <c r="AMG39" s="75" t="n"/>
+      <c r="AMH39" s="75" t="n"/>
+      <c r="AMI39" s="75" t="n"/>
+      <c r="AMJ39" s="75" t="n"/>
     </row>
     <row r="40" ht="17.25" customFormat="1" customHeight="1" s="50">
       <c r="B40" s="62">
@@ -2335,12 +2338,12 @@
       <c r="O40" s="68" t="n"/>
       <c r="P40" s="61" t="n"/>
       <c r="Q40" s="61" t="n"/>
-      <c r="AME40" s="42" t="n"/>
-      <c r="AMF40" s="42" t="n"/>
-      <c r="AMG40" s="42" t="n"/>
-      <c r="AMH40" s="42" t="n"/>
-      <c r="AMI40" s="42" t="n"/>
-      <c r="AMJ40" s="42" t="n"/>
+      <c r="AME40" s="75" t="n"/>
+      <c r="AMF40" s="75" t="n"/>
+      <c r="AMG40" s="75" t="n"/>
+      <c r="AMH40" s="75" t="n"/>
+      <c r="AMI40" s="75" t="n"/>
+      <c r="AMJ40" s="75" t="n"/>
     </row>
     <row r="41" ht="17.25" customFormat="1" customHeight="1" s="50">
       <c r="B41" s="62">
@@ -2361,12 +2364,12 @@
       <c r="O41" s="68" t="n"/>
       <c r="P41" s="61" t="n"/>
       <c r="Q41" s="61" t="n"/>
-      <c r="AME41" s="42" t="n"/>
-      <c r="AMF41" s="42" t="n"/>
-      <c r="AMG41" s="42" t="n"/>
-      <c r="AMH41" s="42" t="n"/>
-      <c r="AMI41" s="42" t="n"/>
-      <c r="AMJ41" s="42" t="n"/>
+      <c r="AME41" s="75" t="n"/>
+      <c r="AMF41" s="75" t="n"/>
+      <c r="AMG41" s="75" t="n"/>
+      <c r="AMH41" s="75" t="n"/>
+      <c r="AMI41" s="75" t="n"/>
+      <c r="AMJ41" s="75" t="n"/>
     </row>
     <row r="42" ht="17.25" customFormat="1" customHeight="1" s="50">
       <c r="B42" s="62">
@@ -2387,12 +2390,12 @@
       <c r="O42" s="68" t="n"/>
       <c r="P42" s="61" t="n"/>
       <c r="Q42" s="61" t="n"/>
-      <c r="AME42" s="42" t="n"/>
-      <c r="AMF42" s="42" t="n"/>
-      <c r="AMG42" s="42" t="n"/>
-      <c r="AMH42" s="42" t="n"/>
-      <c r="AMI42" s="42" t="n"/>
-      <c r="AMJ42" s="42" t="n"/>
+      <c r="AME42" s="75" t="n"/>
+      <c r="AMF42" s="75" t="n"/>
+      <c r="AMG42" s="75" t="n"/>
+      <c r="AMH42" s="75" t="n"/>
+      <c r="AMI42" s="75" t="n"/>
+      <c r="AMJ42" s="75" t="n"/>
     </row>
     <row r="43" ht="17.25" customFormat="1" customHeight="1" s="50">
       <c r="B43" s="62">
@@ -2413,12 +2416,12 @@
       <c r="O43" s="68" t="n"/>
       <c r="P43" s="61" t="n"/>
       <c r="Q43" s="61" t="n"/>
-      <c r="AME43" s="42" t="n"/>
-      <c r="AMF43" s="42" t="n"/>
-      <c r="AMG43" s="42" t="n"/>
-      <c r="AMH43" s="42" t="n"/>
-      <c r="AMI43" s="42" t="n"/>
-      <c r="AMJ43" s="42" t="n"/>
+      <c r="AME43" s="75" t="n"/>
+      <c r="AMF43" s="75" t="n"/>
+      <c r="AMG43" s="75" t="n"/>
+      <c r="AMH43" s="75" t="n"/>
+      <c r="AMI43" s="75" t="n"/>
+      <c r="AMJ43" s="75" t="n"/>
     </row>
     <row r="44" ht="17.25" customFormat="1" customHeight="1" s="50">
       <c r="B44" s="62">
@@ -2439,12 +2442,12 @@
       <c r="O44" s="68" t="n"/>
       <c r="P44" s="61" t="n"/>
       <c r="Q44" s="61" t="n"/>
-      <c r="AME44" s="42" t="n"/>
-      <c r="AMF44" s="42" t="n"/>
-      <c r="AMG44" s="42" t="n"/>
-      <c r="AMH44" s="42" t="n"/>
-      <c r="AMI44" s="42" t="n"/>
-      <c r="AMJ44" s="42" t="n"/>
+      <c r="AME44" s="75" t="n"/>
+      <c r="AMF44" s="75" t="n"/>
+      <c r="AMG44" s="75" t="n"/>
+      <c r="AMH44" s="75" t="n"/>
+      <c r="AMI44" s="75" t="n"/>
+      <c r="AMJ44" s="75" t="n"/>
     </row>
     <row r="45" ht="17.25" customFormat="1" customHeight="1" s="50">
       <c r="B45" s="62">
@@ -2465,12 +2468,12 @@
       <c r="O45" s="68" t="n"/>
       <c r="P45" s="61" t="n"/>
       <c r="Q45" s="61" t="n"/>
-      <c r="AME45" s="42" t="n"/>
-      <c r="AMF45" s="42" t="n"/>
-      <c r="AMG45" s="42" t="n"/>
-      <c r="AMH45" s="42" t="n"/>
-      <c r="AMI45" s="42" t="n"/>
-      <c r="AMJ45" s="42" t="n"/>
+      <c r="AME45" s="75" t="n"/>
+      <c r="AMF45" s="75" t="n"/>
+      <c r="AMG45" s="75" t="n"/>
+      <c r="AMH45" s="75" t="n"/>
+      <c r="AMI45" s="75" t="n"/>
+      <c r="AMJ45" s="75" t="n"/>
     </row>
     <row r="46" ht="12.75" customHeight="1" s="69">
       <c r="F46" s="65" t="n"/>
@@ -13965,18 +13968,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I246"/>
+  <dimension ref="A1:R1700"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.43359375" defaultRowHeight="12.75" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="24.67" customWidth="1" style="42" min="1" max="1"/>
-    <col width="49.34" customWidth="1" style="42" min="2" max="2"/>
-    <col width="37.18" customWidth="1" style="42" min="4" max="4"/>
-    <col width="24.58" customWidth="1" style="42" min="5" max="5"/>
-    <col width="27.73" customWidth="1" style="42" min="6" max="6"/>
-    <col width="19.5" customWidth="1" style="42" min="7" max="7"/>
-    <col width="71.98" customWidth="1" style="42" min="8" max="8"/>
-    <col width="34.52" customWidth="1" style="42" min="9" max="9"/>
-    <col width="11.52" customWidth="1" style="42" min="1024" max="1024"/>
+    <col width="24.67" customWidth="1" style="75" min="1" max="1"/>
+    <col width="49.34" customWidth="1" style="75" min="2" max="2"/>
+    <col width="37.18" customWidth="1" style="75" min="4" max="4"/>
+    <col width="24.58" customWidth="1" style="75" min="5" max="5"/>
+    <col width="27.73" customWidth="1" style="75" min="6" max="6"/>
+    <col width="19.5" customWidth="1" style="75" min="7" max="7"/>
+    <col width="71.98" customWidth="1" style="75" min="8" max="8"/>
+    <col width="34.52" customWidth="1" style="75" min="9" max="9"/>
+    <col width="20" customWidth="1" style="69" min="18" max="18"/>
+    <col width="11.52" customWidth="1" style="75" min="1024" max="1024"/>
   </cols>
   <sheetData>
     <row r="1" ht="12.75" customHeight="1" s="69">
@@ -14016,24 +14020,29 @@
           <t>Тип разрешительной документации</t>
         </is>
       </c>
+      <c r="R1" s="75" t="inlineStr">
+        <is>
+          <t>Вес в граммах</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="13.5" customHeight="1" s="69">
-      <c r="D2" s="42" t="inlineStr">
+      <c r="D2" s="75" t="inlineStr">
         <is>
           <t>АРАФАТКА</t>
         </is>
       </c>
-      <c r="E2" s="42" t="inlineStr">
+      <c r="E2" s="75" t="inlineStr">
         <is>
           <t>БЕЖЕВЫЙ</t>
         </is>
       </c>
-      <c r="F2" s="42" t="inlineStr">
+      <c r="F2" s="75" t="inlineStr">
         <is>
           <t>Жен.</t>
         </is>
       </c>
-      <c r="G2" s="42" t="inlineStr">
+      <c r="G2" s="75" t="inlineStr">
         <is>
           <t>РОССИЯ</t>
         </is>
@@ -14060,22 +14069,22 @@
           <t>Значение атрибута</t>
         </is>
       </c>
-      <c r="D3" s="42" t="inlineStr">
+      <c r="D3" s="75" t="inlineStr">
         <is>
           <t>БАБОЧКА</t>
         </is>
       </c>
-      <c r="E3" s="42" t="inlineStr">
+      <c r="E3" s="75" t="inlineStr">
         <is>
           <t>БЕЖЕВЫЙ МЕЛАНЖ</t>
         </is>
       </c>
-      <c r="F3" s="42" t="inlineStr">
+      <c r="F3" s="75" t="inlineStr">
         <is>
           <t>Муж.</t>
         </is>
       </c>
-      <c r="G3" s="42" t="inlineStr">
+      <c r="G3" s="75" t="inlineStr">
         <is>
           <t>МЕЖДУНАРОДНЫЙ</t>
         </is>
@@ -14092,22 +14101,22 @@
       </c>
     </row>
     <row r="4" ht="13.5" customHeight="1" s="69">
-      <c r="D4" s="42" t="inlineStr">
+      <c r="D4" s="75" t="inlineStr">
         <is>
           <t>БАНТ</t>
         </is>
       </c>
-      <c r="E4" s="42" t="inlineStr">
+      <c r="E4" s="75" t="inlineStr">
         <is>
           <t>БЕЖЕВЫЙ/ЗЕЛЕНЫЙ</t>
         </is>
       </c>
-      <c r="F4" s="42" t="inlineStr">
+      <c r="F4" s="75" t="inlineStr">
         <is>
           <t>Унисекс</t>
         </is>
       </c>
-      <c r="G4" s="42" t="inlineStr">
+      <c r="G4" s="75" t="inlineStr">
         <is>
           <t>ДЛИНА-ШИРИНА</t>
         </is>
@@ -14119,17 +14128,17 @@
       </c>
     </row>
     <row r="5" ht="13.5" customHeight="1" s="69">
-      <c r="D5" s="42" t="inlineStr">
+      <c r="D5" s="75" t="inlineStr">
         <is>
           <t>БАСКА</t>
         </is>
       </c>
-      <c r="E5" s="42" t="inlineStr">
+      <c r="E5" s="75" t="inlineStr">
         <is>
           <t>БЕЖЕВЫЙ/СИНИЙ</t>
         </is>
       </c>
-      <c r="F5" s="42" t="inlineStr">
+      <c r="F5" s="75" t="inlineStr">
         <is>
           <t>Детск.</t>
         </is>
@@ -14140,13 +14149,13 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="13.5" customHeight="1" s="69">
-      <c r="D6" s="42" t="inlineStr">
+    <row r="6" ht="160" customHeight="1" s="69">
+      <c r="D6" s="75" t="inlineStr">
         <is>
           <t>БАФФ</t>
         </is>
       </c>
-      <c r="E6" s="42" t="inlineStr">
+      <c r="E6" s="75" t="inlineStr">
         <is>
           <t>БЕЛО-ЗЕЛЕНЫЙ</t>
         </is>
@@ -14156,14 +14165,19 @@
           <t>АЛАНДСКИЕ ОСТРОВА</t>
         </is>
       </c>
+      <c r="R6" s="86" t="inlineStr">
+        <is>
+          <t>Обязательное поле: общий вес позиции, целое число больше 0. Просьба указать актуальный вес товара в ГРАММАХ для отчетности РОСПРИРОДНАДЗОР.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="13.5" customHeight="1" s="69">
-      <c r="D7" s="42" t="inlineStr">
+      <c r="D7" s="75" t="inlineStr">
         <is>
           <t>ВОРОТНИК</t>
         </is>
       </c>
-      <c r="E7" s="42" t="inlineStr">
+      <c r="E7" s="75" t="inlineStr">
         <is>
           <t>БЕЛО-КОРИЧНЕВЫЙ</t>
         </is>
@@ -14175,12 +14189,12 @@
       </c>
     </row>
     <row r="8" ht="13.5" customHeight="1" s="69">
-      <c r="D8" s="42" t="inlineStr">
+      <c r="D8" s="75" t="inlineStr">
         <is>
           <t>ВОРОТНИК-ГАЛСТУК</t>
         </is>
       </c>
-      <c r="E8" s="42" t="inlineStr">
+      <c r="E8" s="75" t="inlineStr">
         <is>
           <t>БЕЛО-РОЗОВЫЙ</t>
         </is>
@@ -14192,12 +14206,12 @@
       </c>
     </row>
     <row r="9" ht="13.5" customHeight="1" s="69">
-      <c r="D9" s="42" t="inlineStr">
+      <c r="D9" s="75" t="inlineStr">
         <is>
           <t>ВУАЛЬ</t>
         </is>
       </c>
-      <c r="E9" s="42" t="inlineStr">
+      <c r="E9" s="75" t="inlineStr">
         <is>
           <t>БЕЛЫЙ</t>
         </is>
@@ -14209,12 +14223,12 @@
       </c>
     </row>
     <row r="10" ht="13.5" customHeight="1" s="69">
-      <c r="D10" s="42" t="inlineStr">
+      <c r="D10" s="75" t="inlineStr">
         <is>
           <t>ГАЛСТУК</t>
         </is>
       </c>
-      <c r="E10" s="42" t="inlineStr">
+      <c r="E10" s="75" t="inlineStr">
         <is>
           <t>БЕЛЫЙ/БЕЖЕВЫЙ</t>
         </is>
@@ -14226,12 +14240,12 @@
       </c>
     </row>
     <row r="11" ht="13.5" customHeight="1" s="69">
-      <c r="D11" s="42" t="inlineStr">
+      <c r="D11" s="75" t="inlineStr">
         <is>
           <t>ГАЛСТУК-БАБОЧКА</t>
         </is>
       </c>
-      <c r="E11" s="42" t="inlineStr">
+      <c r="E11" s="75" t="inlineStr">
         <is>
           <t>БЕЛЫЙ/СЕРЫЙ</t>
         </is>
@@ -14243,12 +14257,12 @@
       </c>
     </row>
     <row r="12" ht="13.5" customHeight="1" s="69">
-      <c r="D12" s="42" t="inlineStr">
+      <c r="D12" s="75" t="inlineStr">
         <is>
           <t>ГЕЙТОР</t>
         </is>
       </c>
-      <c r="E12" s="42" t="inlineStr">
+      <c r="E12" s="75" t="inlineStr">
         <is>
           <t>БЕЛЫЙ/СИНИЙ</t>
         </is>
@@ -14260,12 +14274,12 @@
       </c>
     </row>
     <row r="13" ht="13.5" customHeight="1" s="69">
-      <c r="D13" s="42" t="inlineStr">
+      <c r="D13" s="75" t="inlineStr">
         <is>
           <t>ГОРЖЕТКА</t>
         </is>
       </c>
-      <c r="E13" s="42" t="inlineStr">
+      <c r="E13" s="75" t="inlineStr">
         <is>
           <t>БИРЮЗОВЫЙ</t>
         </is>
@@ -14277,12 +14291,12 @@
       </c>
     </row>
     <row r="14" ht="13.5" customHeight="1" s="69">
-      <c r="D14" s="42" t="inlineStr">
+      <c r="D14" s="75" t="inlineStr">
         <is>
           <t>ГЮЙС</t>
         </is>
       </c>
-      <c r="E14" s="42" t="inlineStr">
+      <c r="E14" s="75" t="inlineStr">
         <is>
           <t>БОРДОВО-РЫЖИЙ</t>
         </is>
@@ -14294,12 +14308,12 @@
       </c>
     </row>
     <row r="15" ht="13.5" customHeight="1" s="69">
-      <c r="D15" s="42" t="inlineStr">
+      <c r="D15" s="75" t="inlineStr">
         <is>
           <t>ЖАБО</t>
         </is>
       </c>
-      <c r="E15" s="42" t="inlineStr">
+      <c r="E15" s="75" t="inlineStr">
         <is>
           <t>БОРДОВЫЙ</t>
         </is>
@@ -14311,12 +14325,12 @@
       </c>
     </row>
     <row r="16" ht="13.5" customHeight="1" s="69">
-      <c r="D16" s="42" t="inlineStr">
+      <c r="D16" s="75" t="inlineStr">
         <is>
           <t>КАШНЕ</t>
         </is>
       </c>
-      <c r="E16" s="42" t="inlineStr">
+      <c r="E16" s="75" t="inlineStr">
         <is>
           <t>БРОНЗОВЫЙ</t>
         </is>
@@ -14328,12 +14342,12 @@
       </c>
     </row>
     <row r="17" ht="13.5" customHeight="1" s="69">
-      <c r="D17" s="42" t="inlineStr">
+      <c r="D17" s="75" t="inlineStr">
         <is>
           <t>МАНИШКА</t>
         </is>
       </c>
-      <c r="E17" s="42" t="inlineStr">
+      <c r="E17" s="75" t="inlineStr">
         <is>
           <t>ВАНИЛЬ</t>
         </is>
@@ -14345,12 +14359,12 @@
       </c>
     </row>
     <row r="18" ht="13.5" customHeight="1" s="69">
-      <c r="D18" s="42" t="inlineStr">
+      <c r="D18" s="75" t="inlineStr">
         <is>
           <t>МАНТИЛЬЯ</t>
         </is>
       </c>
-      <c r="E18" s="42" t="inlineStr">
+      <c r="E18" s="75" t="inlineStr">
         <is>
           <t>ВИШНЯ</t>
         </is>
@@ -14362,12 +14376,12 @@
       </c>
     </row>
     <row r="19" ht="13.5" customHeight="1" s="69">
-      <c r="D19" s="42" t="inlineStr">
+      <c r="D19" s="75" t="inlineStr">
         <is>
           <t>МАСКА</t>
         </is>
       </c>
-      <c r="E19" s="42" t="inlineStr">
+      <c r="E19" s="75" t="inlineStr">
         <is>
           <t>ГОЛУБОЙ</t>
         </is>
@@ -14379,12 +14393,12 @@
       </c>
     </row>
     <row r="20" ht="13.5" customHeight="1" s="69">
-      <c r="D20" s="42" t="inlineStr">
+      <c r="D20" s="75" t="inlineStr">
         <is>
           <t>НАГРУДНИК</t>
         </is>
       </c>
-      <c r="E20" s="42" t="inlineStr">
+      <c r="E20" s="75" t="inlineStr">
         <is>
           <t>ГОРЧИЧНЫЙ</t>
         </is>
@@ -14396,12 +14410,12 @@
       </c>
     </row>
     <row r="21" ht="13.5" customHeight="1" s="69">
-      <c r="D21" s="42" t="inlineStr">
+      <c r="D21" s="75" t="inlineStr">
         <is>
           <t>НАМАЗНИК</t>
         </is>
       </c>
-      <c r="E21" s="42" t="inlineStr">
+      <c r="E21" s="75" t="inlineStr">
         <is>
           <t>ГРАФИТОВЫЙ</t>
         </is>
@@ -14413,12 +14427,12 @@
       </c>
     </row>
     <row r="22" ht="13.5" customHeight="1" s="69">
-      <c r="D22" s="42" t="inlineStr">
+      <c r="D22" s="75" t="inlineStr">
         <is>
           <t>ПАЛАНТИН</t>
         </is>
       </c>
-      <c r="E22" s="42" t="inlineStr">
+      <c r="E22" s="75" t="inlineStr">
         <is>
           <t>ЖЁЛТЫЙ</t>
         </is>
@@ -14430,12 +14444,12 @@
       </c>
     </row>
     <row r="23" ht="13.5" customHeight="1" s="69">
-      <c r="D23" s="42" t="inlineStr">
+      <c r="D23" s="75" t="inlineStr">
         <is>
           <t>ПАРЕО</t>
         </is>
       </c>
-      <c r="E23" s="42" t="inlineStr">
+      <c r="E23" s="75" t="inlineStr">
         <is>
           <t>ЗЕЛЁНЫЙ</t>
         </is>
@@ -14447,12 +14461,12 @@
       </c>
     </row>
     <row r="24" ht="13.5" customHeight="1" s="69">
-      <c r="D24" s="42" t="inlineStr">
+      <c r="D24" s="75" t="inlineStr">
         <is>
           <t>ПАШЕ</t>
         </is>
       </c>
-      <c r="E24" s="42" t="inlineStr">
+      <c r="E24" s="75" t="inlineStr">
         <is>
           <t>ЗОЛОТИСТЫЙ</t>
         </is>
@@ -14464,12 +14478,12 @@
       </c>
     </row>
     <row r="25" ht="13.5" customHeight="1" s="69">
-      <c r="D25" s="42" t="inlineStr">
+      <c r="D25" s="75" t="inlineStr">
         <is>
           <t>ПЕЛЕРИНА</t>
         </is>
       </c>
-      <c r="E25" s="42" t="inlineStr">
+      <c r="E25" s="75" t="inlineStr">
         <is>
           <t>ЗОЛОТОЙ</t>
         </is>
@@ -14481,12 +14495,12 @@
       </c>
     </row>
     <row r="26" ht="13.5" customHeight="1" s="69">
-      <c r="D26" s="42" t="inlineStr">
+      <c r="D26" s="75" t="inlineStr">
         <is>
           <t>ПЛАТОК ГОЛОВНОЙ</t>
         </is>
       </c>
-      <c r="E26" s="42" t="inlineStr">
+      <c r="E26" s="75" t="inlineStr">
         <is>
           <t>ИЗУМРУДНЫЙ</t>
         </is>
@@ -14498,12 +14512,12 @@
       </c>
     </row>
     <row r="27" ht="13.5" customHeight="1" s="69">
-      <c r="D27" s="42" t="inlineStr">
+      <c r="D27" s="75" t="inlineStr">
         <is>
           <t>ПЛАТОК НОСОВОЙ</t>
         </is>
       </c>
-      <c r="E27" s="42" t="inlineStr">
+      <c r="E27" s="75" t="inlineStr">
         <is>
           <t>КАПУЧИНО</t>
         </is>
@@ -14515,12 +14529,12 @@
       </c>
     </row>
     <row r="28" ht="13.5" customHeight="1" s="69">
-      <c r="D28" s="42" t="inlineStr">
+      <c r="D28" s="75" t="inlineStr">
         <is>
           <t>ПЛАТОК ШЕЙНЫЙ</t>
         </is>
       </c>
-      <c r="E28" s="42" t="inlineStr">
+      <c r="E28" s="75" t="inlineStr">
         <is>
           <t>КИРПИЧНЫЙ</t>
         </is>
@@ -14532,12 +14546,12 @@
       </c>
     </row>
     <row r="29" ht="13.5" customHeight="1" s="69">
-      <c r="D29" s="42" t="inlineStr">
+      <c r="D29" s="75" t="inlineStr">
         <is>
           <t>ПОВЯЗКА НА ГОЛОВУ</t>
         </is>
       </c>
-      <c r="E29" s="42" t="inlineStr">
+      <c r="E29" s="75" t="inlineStr">
         <is>
           <t>КОРАЛЛОВЫЙ</t>
         </is>
@@ -14549,12 +14563,12 @@
       </c>
     </row>
     <row r="30" ht="13.5" customHeight="1" s="69">
-      <c r="D30" s="42" t="inlineStr">
+      <c r="D30" s="75" t="inlineStr">
         <is>
           <t>ПОДТЯЖКИ</t>
         </is>
       </c>
-      <c r="E30" s="42" t="inlineStr">
+      <c r="E30" s="75" t="inlineStr">
         <is>
           <t>КОРИЧНЕВЫЙ</t>
         </is>
@@ -14566,12 +14580,12 @@
       </c>
     </row>
     <row r="31" ht="13.5" customHeight="1" s="69">
-      <c r="D31" s="42" t="inlineStr">
+      <c r="D31" s="75" t="inlineStr">
         <is>
           <t>ПОРТУПЕЯ</t>
         </is>
       </c>
-      <c r="E31" s="42" t="inlineStr">
+      <c r="E31" s="75" t="inlineStr">
         <is>
           <t>КОФЕЙНЫЙ</t>
         </is>
@@ -14583,12 +14597,12 @@
       </c>
     </row>
     <row r="32" ht="13.5" customHeight="1" s="69">
-      <c r="D32" s="42" t="inlineStr">
+      <c r="D32" s="75" t="inlineStr">
         <is>
           <t>ПОЯС</t>
         </is>
       </c>
-      <c r="E32" s="42" t="inlineStr">
+      <c r="E32" s="75" t="inlineStr">
         <is>
           <t>КРАСНО-КОРИЧНЕВЫЙ</t>
         </is>
@@ -14600,12 +14614,12 @@
       </c>
     </row>
     <row r="33" ht="13.5" customHeight="1" s="69">
-      <c r="D33" s="42" t="inlineStr">
+      <c r="D33" s="75" t="inlineStr">
         <is>
           <t>РЕМЕНЬ</t>
         </is>
       </c>
-      <c r="E33" s="42" t="inlineStr">
+      <c r="E33" s="75" t="inlineStr">
         <is>
           <t>КРАСНЫЙ</t>
         </is>
@@ -14617,12 +14631,12 @@
       </c>
     </row>
     <row r="34" ht="13.5" customHeight="1" s="69">
-      <c r="D34" s="42" t="inlineStr">
+      <c r="D34" s="75" t="inlineStr">
         <is>
           <t>РУКАВА</t>
         </is>
       </c>
-      <c r="E34" s="42" t="inlineStr">
+      <c r="E34" s="75" t="inlineStr">
         <is>
           <t>КРЕМОВЫЙ</t>
         </is>
@@ -14634,12 +14648,12 @@
       </c>
     </row>
     <row r="35" ht="13.5" customHeight="1" s="69">
-      <c r="D35" s="42" t="inlineStr">
+      <c r="D35" s="75" t="inlineStr">
         <is>
           <t>ХИДЖАБ</t>
         </is>
       </c>
-      <c r="E35" s="42" t="inlineStr">
+      <c r="E35" s="75" t="inlineStr">
         <is>
           <t>ЛАВАНДОВЫЙ</t>
         </is>
@@ -14651,12 +14665,12 @@
       </c>
     </row>
     <row r="36" ht="13.5" customHeight="1" s="69">
-      <c r="D36" s="42" t="inlineStr">
+      <c r="D36" s="75" t="inlineStr">
         <is>
           <t>ШАЛЬ</t>
         </is>
       </c>
-      <c r="E36" s="42" t="inlineStr">
+      <c r="E36" s="75" t="inlineStr">
         <is>
           <t>ЛАЙМ</t>
         </is>
@@ -14668,12 +14682,12 @@
       </c>
     </row>
     <row r="37" ht="13.5" customHeight="1" s="69">
-      <c r="D37" s="42" t="inlineStr">
+      <c r="D37" s="75" t="inlineStr">
         <is>
           <t>ШАРФ-СНУД</t>
         </is>
       </c>
-      <c r="E37" s="42" t="inlineStr">
+      <c r="E37" s="75" t="inlineStr">
         <is>
           <t>ЛЕОПАРД</t>
         </is>
@@ -14690,7 +14704,7 @@
           <t>ГАЛСТУК-БАНТ</t>
         </is>
       </c>
-      <c r="E38" s="42" t="inlineStr">
+      <c r="E38" s="75" t="inlineStr">
         <is>
           <t>МАЛИНОВЫЙ</t>
         </is>
@@ -14702,7 +14716,7 @@
       </c>
     </row>
     <row r="39" ht="13.5" customHeight="1" s="69">
-      <c r="E39" s="42" t="inlineStr">
+      <c r="E39" s="75" t="inlineStr">
         <is>
           <t>МЕДНЫЙ</t>
         </is>
@@ -14714,7 +14728,7 @@
       </c>
     </row>
     <row r="40" ht="13.5" customHeight="1" s="69">
-      <c r="E40" s="42" t="inlineStr">
+      <c r="E40" s="75" t="inlineStr">
         <is>
           <t>МОЛОЧНЫЙ</t>
         </is>
@@ -14726,7 +14740,7 @@
       </c>
     </row>
     <row r="41" ht="13.5" customHeight="1" s="69">
-      <c r="E41" s="42" t="inlineStr">
+      <c r="E41" s="75" t="inlineStr">
         <is>
           <t>МЯТНЫЙ</t>
         </is>
@@ -14738,7 +14752,7 @@
       </c>
     </row>
     <row r="42" ht="13.5" customHeight="1" s="69">
-      <c r="E42" s="42" t="inlineStr">
+      <c r="E42" s="75" t="inlineStr">
         <is>
           <t>НАТУРАЛЬНЫЙ</t>
         </is>
@@ -14750,7 +14764,7 @@
       </c>
     </row>
     <row r="43" ht="13.5" customHeight="1" s="69">
-      <c r="E43" s="42" t="inlineStr">
+      <c r="E43" s="75" t="inlineStr">
         <is>
           <t>НИКЕЛЬ</t>
         </is>
@@ -14762,7 +14776,7 @@
       </c>
     </row>
     <row r="44" ht="13.5" customHeight="1" s="69">
-      <c r="E44" s="42" t="inlineStr">
+      <c r="E44" s="75" t="inlineStr">
         <is>
           <t>ОЛИВКОВО-БЕЛЫЙ</t>
         </is>
@@ -14774,7 +14788,7 @@
       </c>
     </row>
     <row r="45" ht="13.5" customHeight="1" s="69">
-      <c r="E45" s="42" t="inlineStr">
+      <c r="E45" s="75" t="inlineStr">
         <is>
           <t>ОЛИВКОВЫЙ</t>
         </is>
@@ -14786,7 +14800,7 @@
       </c>
     </row>
     <row r="46" ht="13.5" customHeight="1" s="69">
-      <c r="E46" s="42" t="inlineStr">
+      <c r="E46" s="75" t="inlineStr">
         <is>
           <t>ОРАНЖЕВЫЙ</t>
         </is>
@@ -14798,7 +14812,7 @@
       </c>
     </row>
     <row r="47" ht="13.5" customHeight="1" s="69">
-      <c r="E47" s="42" t="inlineStr">
+      <c r="E47" s="75" t="inlineStr">
         <is>
           <t>ПЕРЛАМУТРОВЫЙ</t>
         </is>
@@ -14810,7 +14824,7 @@
       </c>
     </row>
     <row r="48" ht="13.5" customHeight="1" s="69">
-      <c r="E48" s="42" t="inlineStr">
+      <c r="E48" s="75" t="inlineStr">
         <is>
           <t>ПЕРСИКОВЫЙ</t>
         </is>
@@ -14822,7 +14836,7 @@
       </c>
     </row>
     <row r="49" ht="13.5" customHeight="1" s="69">
-      <c r="E49" s="42" t="inlineStr">
+      <c r="E49" s="75" t="inlineStr">
         <is>
           <t>ПЕСОЧНЫЙ</t>
         </is>
@@ -14834,7 +14848,7 @@
       </c>
     </row>
     <row r="50" ht="13.5" customHeight="1" s="69">
-      <c r="E50" s="42" t="inlineStr">
+      <c r="E50" s="75" t="inlineStr">
         <is>
           <t>ПРОЗРАЧНЫЙ</t>
         </is>
@@ -14846,7 +14860,7 @@
       </c>
     </row>
     <row r="51" ht="13.5" customHeight="1" s="69">
-      <c r="E51" s="42" t="inlineStr">
+      <c r="E51" s="75" t="inlineStr">
         <is>
           <t>ПУРПУРНЫЙ</t>
         </is>
@@ -14858,7 +14872,7 @@
       </c>
     </row>
     <row r="52" ht="13.5" customHeight="1" s="69">
-      <c r="E52" s="42" t="inlineStr">
+      <c r="E52" s="75" t="inlineStr">
         <is>
           <t>РАЗНОЦВЕТНЫЙ</t>
         </is>
@@ -14870,7 +14884,7 @@
       </c>
     </row>
     <row r="53" ht="13.5" customHeight="1" s="69">
-      <c r="E53" s="42" t="inlineStr">
+      <c r="E53" s="75" t="inlineStr">
         <is>
           <t>РОЗОВО-БЕЖЕВЫЙ</t>
         </is>
@@ -14882,7 +14896,7 @@
       </c>
     </row>
     <row r="54" ht="13.5" customHeight="1" s="69">
-      <c r="E54" s="42" t="inlineStr">
+      <c r="E54" s="75" t="inlineStr">
         <is>
           <t>РОЗОВЫЙ</t>
         </is>
@@ -14894,7 +14908,7 @@
       </c>
     </row>
     <row r="55" ht="13.5" customHeight="1" s="69">
-      <c r="E55" s="42" t="inlineStr">
+      <c r="E55" s="75" t="inlineStr">
         <is>
           <t>РЫЖЕ-КОРИЧНЕВЫЙ</t>
         </is>
@@ -14906,7 +14920,7 @@
       </c>
     </row>
     <row r="56" ht="13.5" customHeight="1" s="69">
-      <c r="E56" s="42" t="inlineStr">
+      <c r="E56" s="75" t="inlineStr">
         <is>
           <t>РЫЖИЙ</t>
         </is>
@@ -14918,7 +14932,7 @@
       </c>
     </row>
     <row r="57" ht="13.5" customHeight="1" s="69">
-      <c r="E57" s="42" t="inlineStr">
+      <c r="E57" s="75" t="inlineStr">
         <is>
           <t>САЛАТОВЫЙ</t>
         </is>
@@ -14930,7 +14944,7 @@
       </c>
     </row>
     <row r="58" ht="13.5" customHeight="1" s="69">
-      <c r="E58" s="42" t="inlineStr">
+      <c r="E58" s="75" t="inlineStr">
         <is>
           <t>СВЕТЛО-БЕЖЕВЫЙ</t>
         </is>
@@ -14942,7 +14956,7 @@
       </c>
     </row>
     <row r="59" ht="13.5" customHeight="1" s="69">
-      <c r="E59" s="42" t="inlineStr">
+      <c r="E59" s="75" t="inlineStr">
         <is>
           <t>СВЕТЛО-ЗЕЛЕНЫЙ</t>
         </is>
@@ -14954,7 +14968,7 @@
       </c>
     </row>
     <row r="60" ht="13.5" customHeight="1" s="69">
-      <c r="E60" s="42" t="inlineStr">
+      <c r="E60" s="75" t="inlineStr">
         <is>
           <t>СВЕТЛО-КОРИЧНЕВЫЙ</t>
         </is>
@@ -14966,7 +14980,7 @@
       </c>
     </row>
     <row r="61" ht="13.5" customHeight="1" s="69">
-      <c r="E61" s="42" t="inlineStr">
+      <c r="E61" s="75" t="inlineStr">
         <is>
           <t>СВЕТЛО-РОЗОВЫЙ</t>
         </is>
@@ -14978,7 +14992,7 @@
       </c>
     </row>
     <row r="62" ht="13.5" customHeight="1" s="69">
-      <c r="E62" s="42" t="inlineStr">
+      <c r="E62" s="75" t="inlineStr">
         <is>
           <t>СВЕТЛО-СЕРЫЙ</t>
         </is>
@@ -14990,7 +15004,7 @@
       </c>
     </row>
     <row r="63" ht="13.5" customHeight="1" s="69">
-      <c r="E63" s="42" t="inlineStr">
+      <c r="E63" s="75" t="inlineStr">
         <is>
           <t>СВЕТЛО-СЕРЫЙ МЕЛАНЖ</t>
         </is>
@@ -15002,7 +15016,7 @@
       </c>
     </row>
     <row r="64" ht="13.5" customHeight="1" s="69">
-      <c r="E64" s="42" t="inlineStr">
+      <c r="E64" s="75" t="inlineStr">
         <is>
           <t>СВЕТЛО-СИНИЙ</t>
         </is>
@@ -15014,7 +15028,7 @@
       </c>
     </row>
     <row r="65" ht="13.5" customHeight="1" s="69">
-      <c r="E65" s="42" t="inlineStr">
+      <c r="E65" s="75" t="inlineStr">
         <is>
           <t>СВЕТЛО-ФИОЛЕТОВЫЙ</t>
         </is>
@@ -15026,7 +15040,7 @@
       </c>
     </row>
     <row r="66" ht="13.5" customHeight="1" s="69">
-      <c r="E66" s="42" t="inlineStr">
+      <c r="E66" s="75" t="inlineStr">
         <is>
           <t>СЕРЕБРЯНЫЙ</t>
         </is>
@@ -15038,7 +15052,7 @@
       </c>
     </row>
     <row r="67" ht="13.5" customHeight="1" s="69">
-      <c r="E67" s="42" t="inlineStr">
+      <c r="E67" s="75" t="inlineStr">
         <is>
           <t>СЕРО-БЕЖЕВЫЙ</t>
         </is>
@@ -15050,7 +15064,7 @@
       </c>
     </row>
     <row r="68" ht="13.5" customHeight="1" s="69">
-      <c r="E68" s="42" t="inlineStr">
+      <c r="E68" s="75" t="inlineStr">
         <is>
           <t>СЕРО-ГОЛУБОЙ</t>
         </is>
@@ -15062,7 +15076,7 @@
       </c>
     </row>
     <row r="69" ht="13.5" customHeight="1" s="69">
-      <c r="E69" s="42" t="inlineStr">
+      <c r="E69" s="75" t="inlineStr">
         <is>
           <t>СЕРО-ЖЕЛТЫЙ</t>
         </is>
@@ -15074,7 +15088,7 @@
       </c>
     </row>
     <row r="70" ht="13.5" customHeight="1" s="69">
-      <c r="E70" s="42" t="inlineStr">
+      <c r="E70" s="75" t="inlineStr">
         <is>
           <t>СЕРЫЙ</t>
         </is>
@@ -15086,7 +15100,7 @@
       </c>
     </row>
     <row r="71" ht="13.5" customHeight="1" s="69">
-      <c r="E71" s="42" t="inlineStr">
+      <c r="E71" s="75" t="inlineStr">
         <is>
           <t>СЕРЫЙ МЕЛАНЖ</t>
         </is>
@@ -15098,7 +15112,7 @@
       </c>
     </row>
     <row r="72" ht="13.5" customHeight="1" s="69">
-      <c r="E72" s="42" t="inlineStr">
+      <c r="E72" s="75" t="inlineStr">
         <is>
           <t>СИНИЙ</t>
         </is>
@@ -15110,7 +15124,7 @@
       </c>
     </row>
     <row r="73" ht="13.5" customHeight="1" s="69">
-      <c r="E73" s="42" t="inlineStr">
+      <c r="E73" s="75" t="inlineStr">
         <is>
           <t>СИРЕНЕВЫЙ/ЛИЛОВЫЙ</t>
         </is>
@@ -15122,7 +15136,7 @@
       </c>
     </row>
     <row r="74" ht="13.5" customHeight="1" s="69">
-      <c r="E74" s="42" t="inlineStr">
+      <c r="E74" s="75" t="inlineStr">
         <is>
           <t>СЛИВОВЫЙ</t>
         </is>
@@ -15134,7 +15148,7 @@
       </c>
     </row>
     <row r="75" ht="13.5" customHeight="1" s="69">
-      <c r="E75" s="42" t="inlineStr">
+      <c r="E75" s="75" t="inlineStr">
         <is>
           <t>СЛОНОВАЯ КОСТЬ</t>
         </is>
@@ -15146,7 +15160,7 @@
       </c>
     </row>
     <row r="76" ht="13.5" customHeight="1" s="69">
-      <c r="E76" s="42" t="inlineStr">
+      <c r="E76" s="75" t="inlineStr">
         <is>
           <t>ТЕМНО-БЕЖЕВЫЙ</t>
         </is>
@@ -15158,7 +15172,7 @@
       </c>
     </row>
     <row r="77" ht="13.5" customHeight="1" s="69">
-      <c r="E77" s="42" t="inlineStr">
+      <c r="E77" s="75" t="inlineStr">
         <is>
           <t>ТЕМНО-ЗЕЛЕНЫЙ</t>
         </is>
@@ -15170,7 +15184,7 @@
       </c>
     </row>
     <row r="78" ht="13.5" customHeight="1" s="69">
-      <c r="E78" s="42" t="inlineStr">
+      <c r="E78" s="75" t="inlineStr">
         <is>
           <t>ТЕМНО-КОРИЧНЕВЫЙ</t>
         </is>
@@ -15182,7 +15196,7 @@
       </c>
     </row>
     <row r="79" ht="13.5" customHeight="1" s="69">
-      <c r="E79" s="42" t="inlineStr">
+      <c r="E79" s="75" t="inlineStr">
         <is>
           <t>ТЕМНО-РОЗОВЫЙ</t>
         </is>
@@ -15194,7 +15208,7 @@
       </c>
     </row>
     <row r="80" ht="13.5" customHeight="1" s="69">
-      <c r="E80" s="42" t="inlineStr">
+      <c r="E80" s="75" t="inlineStr">
         <is>
           <t>ТЕМНО-СЕРЫЙ</t>
         </is>
@@ -15206,7 +15220,7 @@
       </c>
     </row>
     <row r="81" ht="13.5" customHeight="1" s="69">
-      <c r="E81" s="42" t="inlineStr">
+      <c r="E81" s="75" t="inlineStr">
         <is>
           <t>ТЕМНО-СЕРЫЙ МЕЛАНЖ</t>
         </is>
@@ -15218,7 +15232,7 @@
       </c>
     </row>
     <row r="82" ht="13.5" customHeight="1" s="69">
-      <c r="E82" s="42" t="inlineStr">
+      <c r="E82" s="75" t="inlineStr">
         <is>
           <t>ТЕМНО-СИНИЙ</t>
         </is>
@@ -15230,7 +15244,7 @@
       </c>
     </row>
     <row r="83" ht="13.5" customHeight="1" s="69">
-      <c r="E83" s="42" t="inlineStr">
+      <c r="E83" s="75" t="inlineStr">
         <is>
           <t>ТЕМНО-ФИОЛЕТОВЫЙ</t>
         </is>
@@ -15242,7 +15256,7 @@
       </c>
     </row>
     <row r="84" ht="13.5" customHeight="1" s="69">
-      <c r="E84" s="42" t="inlineStr">
+      <c r="E84" s="75" t="inlineStr">
         <is>
           <t>ТЕРРАКОТОВЫЙ</t>
         </is>
@@ -15254,7 +15268,7 @@
       </c>
     </row>
     <row r="85" ht="13.5" customHeight="1" s="69">
-      <c r="E85" s="42" t="inlineStr">
+      <c r="E85" s="75" t="inlineStr">
         <is>
           <t>ФИОЛЕТОВЫЙ</t>
         </is>
@@ -15266,7 +15280,7 @@
       </c>
     </row>
     <row r="86" ht="13.5" customHeight="1" s="69">
-      <c r="E86" s="42" t="inlineStr">
+      <c r="E86" s="75" t="inlineStr">
         <is>
           <t>ФИСТАШКОВЫЙ</t>
         </is>
@@ -15278,7 +15292,7 @@
       </c>
     </row>
     <row r="87" ht="13.5" customHeight="1" s="69">
-      <c r="E87" s="42" t="inlineStr">
+      <c r="E87" s="75" t="inlineStr">
         <is>
           <t>ФУКСИЯ</t>
         </is>
@@ -15290,7 +15304,7 @@
       </c>
     </row>
     <row r="88" ht="13.5" customHeight="1" s="69">
-      <c r="E88" s="42" t="inlineStr">
+      <c r="E88" s="75" t="inlineStr">
         <is>
           <t>ХАКИ</t>
         </is>
@@ -15302,7 +15316,7 @@
       </c>
     </row>
     <row r="89" ht="13.5" customHeight="1" s="69">
-      <c r="E89" s="42" t="inlineStr">
+      <c r="E89" s="75" t="inlineStr">
         <is>
           <t>ХАКИ/ОЛИВКОВЫЙ</t>
         </is>
@@ -15314,7 +15328,7 @@
       </c>
     </row>
     <row r="90" ht="13.5" customHeight="1" s="69">
-      <c r="E90" s="42" t="inlineStr">
+      <c r="E90" s="75" t="inlineStr">
         <is>
           <t>ЧЕРНЫЙ</t>
         </is>
@@ -15326,7 +15340,7 @@
       </c>
     </row>
     <row r="91" ht="13.5" customHeight="1" s="69">
-      <c r="E91" s="42" t="inlineStr">
+      <c r="E91" s="75" t="inlineStr">
         <is>
           <t>ЧЕРНЫЙ/БЕЛЫЙ</t>
         </is>
@@ -15338,7 +15352,7 @@
       </c>
     </row>
     <row r="92" ht="13.5" customHeight="1" s="69">
-      <c r="E92" s="42" t="inlineStr">
+      <c r="E92" s="75" t="inlineStr">
         <is>
           <t>ЧЕРНЫЙ/ЗОЛОТИСТЫЙ</t>
         </is>
@@ -15350,7 +15364,7 @@
       </c>
     </row>
     <row r="93" ht="13.5" customHeight="1" s="69">
-      <c r="E93" s="42" t="inlineStr">
+      <c r="E93" s="75" t="inlineStr">
         <is>
           <t>ЧЕРНЫЙ/СЕРЫЙ</t>
         </is>
@@ -15362,7 +15376,7 @@
       </c>
     </row>
     <row r="94" ht="13.5" customHeight="1" s="69">
-      <c r="E94" s="42" t="inlineStr">
+      <c r="E94" s="75" t="inlineStr">
         <is>
           <t>ШОКОЛАДНЫЙ</t>
         </is>
@@ -15374,7 +15388,7 @@
       </c>
     </row>
     <row r="95" ht="13.5" customHeight="1" s="69">
-      <c r="E95" s="42" t="inlineStr">
+      <c r="E95" s="75" t="inlineStr">
         <is>
           <t>СВЕТЛО-ЖЕЛТЫЙ</t>
         </is>
@@ -15386,7 +15400,7 @@
       </c>
     </row>
     <row r="96" ht="13.5" customHeight="1" s="69">
-      <c r="E96" s="42" t="inlineStr">
+      <c r="E96" s="75" t="inlineStr">
         <is>
           <t>ТЕМНО-ЖЕЛТЫЙ</t>
         </is>
@@ -15398,7 +15412,7 @@
       </c>
     </row>
     <row r="97" ht="13.5" customHeight="1" s="69">
-      <c r="E97" s="42" t="inlineStr">
+      <c r="E97" s="75" t="inlineStr">
         <is>
           <t>ЛИЛОВЫЙ</t>
         </is>
@@ -15410,7 +15424,7 @@
       </c>
     </row>
     <row r="98" ht="13.5" customHeight="1" s="69">
-      <c r="E98" s="42" t="inlineStr">
+      <c r="E98" s="75" t="inlineStr">
         <is>
           <t>СЕРЫЙ/ЗЕЛЕНЫЙ</t>
         </is>
@@ -15422,7 +15436,7 @@
       </c>
     </row>
     <row r="99" ht="13.5" customHeight="1" s="69">
-      <c r="E99" s="42" t="inlineStr">
+      <c r="E99" s="75" t="inlineStr">
         <is>
           <t>СИНЕ-ЗЕЛЕНЫЙ</t>
         </is>
@@ -15434,7 +15448,7 @@
       </c>
     </row>
     <row r="100" ht="13.5" customHeight="1" s="69">
-      <c r="E100" s="42" t="inlineStr">
+      <c r="E100" s="75" t="inlineStr">
         <is>
           <t>БЕЛО-ГОЛУБОЙ</t>
         </is>
@@ -15446,7 +15460,7 @@
       </c>
     </row>
     <row r="101" ht="13.5" customHeight="1" s="69">
-      <c r="E101" s="42" t="inlineStr">
+      <c r="E101" s="75" t="inlineStr">
         <is>
           <t>БЕЛО-СИНИЙ</t>
         </is>
@@ -15458,7 +15472,7 @@
       </c>
     </row>
     <row r="102" ht="13.5" customHeight="1" s="69">
-      <c r="E102" s="42" t="inlineStr">
+      <c r="E102" s="75" t="inlineStr">
         <is>
           <t>СВЕТЛО-ГОЛУБОЙ</t>
         </is>
@@ -15470,7 +15484,7 @@
       </c>
     </row>
     <row r="103" ht="13.5" customHeight="1" s="69">
-      <c r="E103" s="42" t="inlineStr">
+      <c r="E103" s="75" t="inlineStr">
         <is>
           <t>ЗЕЛЕНЫЙ МЕЛАНЖ</t>
         </is>
@@ -15482,7 +15496,7 @@
       </c>
     </row>
     <row r="104" ht="13.5" customHeight="1" s="69">
-      <c r="E104" s="42" t="inlineStr">
+      <c r="E104" s="75" t="inlineStr">
         <is>
           <t>ЖЕЛТЫЙ МЕЛАНЖ</t>
         </is>
@@ -15494,7 +15508,7 @@
       </c>
     </row>
     <row r="105" ht="13.5" customHeight="1" s="69">
-      <c r="E105" s="42" t="inlineStr">
+      <c r="E105" s="75" t="inlineStr">
         <is>
           <t>СИНИЙ МЕЛАНЖ</t>
         </is>
@@ -15506,7 +15520,7 @@
       </c>
     </row>
     <row r="106" ht="13.5" customHeight="1" s="69">
-      <c r="E106" s="42" t="inlineStr">
+      <c r="E106" s="75" t="inlineStr">
         <is>
           <t>КРАСНЫЙ МЕЛАНЖ</t>
         </is>
@@ -15518,7 +15532,7 @@
       </c>
     </row>
     <row r="107" ht="13.5" customHeight="1" s="69">
-      <c r="E107" s="42" t="inlineStr">
+      <c r="E107" s="75" t="inlineStr">
         <is>
           <t>РОЗОВЫЙ МЕЛАНЖ</t>
         </is>
@@ -15530,7 +15544,7 @@
       </c>
     </row>
     <row r="108" ht="13.5" customHeight="1" s="69">
-      <c r="E108" s="42" t="inlineStr">
+      <c r="E108" s="75" t="inlineStr">
         <is>
           <t>ФИОЛЕТОВЫЙ МЕЛАНЖ</t>
         </is>
@@ -15542,7 +15556,7 @@
       </c>
     </row>
     <row r="109" ht="13.5" customHeight="1" s="69">
-      <c r="E109" s="42" t="inlineStr">
+      <c r="E109" s="75" t="inlineStr">
         <is>
           <t>ЖЕЛТО-ЗЕЛЕНЫЙ</t>
         </is>
@@ -15554,7 +15568,7 @@
       </c>
     </row>
     <row r="110" ht="13.5" customHeight="1" s="69">
-      <c r="E110" s="42" t="inlineStr">
+      <c r="E110" s="75" t="inlineStr">
         <is>
           <t>МЕЛАНЖ</t>
         </is>
@@ -15566,7 +15580,7 @@
       </c>
     </row>
     <row r="111" ht="13.5" customHeight="1" s="69">
-      <c r="E111" s="42" t="inlineStr">
+      <c r="E111" s="75" t="inlineStr">
         <is>
           <t>СЕРО-ЗЕЛЕНЫЙ</t>
         </is>
@@ -15578,7 +15592,7 @@
       </c>
     </row>
     <row r="112" ht="13.5" customHeight="1" s="69">
-      <c r="E112" s="42" t="inlineStr">
+      <c r="E112" s="75" t="inlineStr">
         <is>
           <t>СЕРО-ЗЕЛЁНЫЙ</t>
         </is>
@@ -15590,7 +15604,7 @@
       </c>
     </row>
     <row r="113" ht="13.5" customHeight="1" s="69">
-      <c r="E113" s="42" t="inlineStr">
+      <c r="E113" s="75" t="inlineStr">
         <is>
           <t>КАМУФЛЯЖНЫЙ</t>
         </is>
@@ -16516,6 +16530,1460 @@
     <row r="246" ht="13.5" customHeight="1" s="69">
       <c r="H246" s="72" t="n"/>
     </row>
+    <row r="247"/>
+    <row r="248"/>
+    <row r="249"/>
+    <row r="250"/>
+    <row r="251"/>
+    <row r="252"/>
+    <row r="253"/>
+    <row r="254"/>
+    <row r="255"/>
+    <row r="256"/>
+    <row r="257"/>
+    <row r="258"/>
+    <row r="259"/>
+    <row r="260"/>
+    <row r="261"/>
+    <row r="262"/>
+    <row r="263"/>
+    <row r="264"/>
+    <row r="265"/>
+    <row r="266"/>
+    <row r="267"/>
+    <row r="268"/>
+    <row r="269"/>
+    <row r="270"/>
+    <row r="271"/>
+    <row r="272"/>
+    <row r="273"/>
+    <row r="274"/>
+    <row r="275"/>
+    <row r="276"/>
+    <row r="277"/>
+    <row r="278"/>
+    <row r="279"/>
+    <row r="280"/>
+    <row r="281"/>
+    <row r="282"/>
+    <row r="283"/>
+    <row r="284"/>
+    <row r="285"/>
+    <row r="286"/>
+    <row r="287"/>
+    <row r="288"/>
+    <row r="289"/>
+    <row r="290"/>
+    <row r="291"/>
+    <row r="292"/>
+    <row r="293"/>
+    <row r="294"/>
+    <row r="295"/>
+    <row r="296"/>
+    <row r="297"/>
+    <row r="298"/>
+    <row r="299"/>
+    <row r="300"/>
+    <row r="301"/>
+    <row r="302"/>
+    <row r="303"/>
+    <row r="304"/>
+    <row r="305"/>
+    <row r="306"/>
+    <row r="307"/>
+    <row r="308"/>
+    <row r="309"/>
+    <row r="310"/>
+    <row r="311"/>
+    <row r="312"/>
+    <row r="313"/>
+    <row r="314"/>
+    <row r="315"/>
+    <row r="316"/>
+    <row r="317"/>
+    <row r="318"/>
+    <row r="319"/>
+    <row r="320"/>
+    <row r="321"/>
+    <row r="322"/>
+    <row r="323"/>
+    <row r="324"/>
+    <row r="325"/>
+    <row r="326"/>
+    <row r="327"/>
+    <row r="328"/>
+    <row r="329"/>
+    <row r="330"/>
+    <row r="331"/>
+    <row r="332"/>
+    <row r="333"/>
+    <row r="334"/>
+    <row r="335"/>
+    <row r="336"/>
+    <row r="337"/>
+    <row r="338"/>
+    <row r="339"/>
+    <row r="340"/>
+    <row r="341"/>
+    <row r="342"/>
+    <row r="343"/>
+    <row r="344"/>
+    <row r="345"/>
+    <row r="346"/>
+    <row r="347"/>
+    <row r="348"/>
+    <row r="349"/>
+    <row r="350"/>
+    <row r="351"/>
+    <row r="352"/>
+    <row r="353"/>
+    <row r="354"/>
+    <row r="355"/>
+    <row r="356"/>
+    <row r="357"/>
+    <row r="358"/>
+    <row r="359"/>
+    <row r="360"/>
+    <row r="361"/>
+    <row r="362"/>
+    <row r="363"/>
+    <row r="364"/>
+    <row r="365"/>
+    <row r="366"/>
+    <row r="367"/>
+    <row r="368"/>
+    <row r="369"/>
+    <row r="370"/>
+    <row r="371"/>
+    <row r="372"/>
+    <row r="373"/>
+    <row r="374"/>
+    <row r="375"/>
+    <row r="376"/>
+    <row r="377"/>
+    <row r="378"/>
+    <row r="379"/>
+    <row r="380"/>
+    <row r="381"/>
+    <row r="382"/>
+    <row r="383"/>
+    <row r="384"/>
+    <row r="385"/>
+    <row r="386"/>
+    <row r="387"/>
+    <row r="388"/>
+    <row r="389"/>
+    <row r="390"/>
+    <row r="391"/>
+    <row r="392"/>
+    <row r="393"/>
+    <row r="394"/>
+    <row r="395"/>
+    <row r="396"/>
+    <row r="397"/>
+    <row r="398"/>
+    <row r="399"/>
+    <row r="400"/>
+    <row r="401"/>
+    <row r="402"/>
+    <row r="403"/>
+    <row r="404"/>
+    <row r="405"/>
+    <row r="406"/>
+    <row r="407"/>
+    <row r="408"/>
+    <row r="409"/>
+    <row r="410"/>
+    <row r="411"/>
+    <row r="412"/>
+    <row r="413"/>
+    <row r="414"/>
+    <row r="415"/>
+    <row r="416"/>
+    <row r="417"/>
+    <row r="418"/>
+    <row r="419"/>
+    <row r="420"/>
+    <row r="421"/>
+    <row r="422"/>
+    <row r="423"/>
+    <row r="424"/>
+    <row r="425"/>
+    <row r="426"/>
+    <row r="427"/>
+    <row r="428"/>
+    <row r="429"/>
+    <row r="430"/>
+    <row r="431"/>
+    <row r="432"/>
+    <row r="433"/>
+    <row r="434"/>
+    <row r="435"/>
+    <row r="436"/>
+    <row r="437"/>
+    <row r="438"/>
+    <row r="439"/>
+    <row r="440"/>
+    <row r="441"/>
+    <row r="442"/>
+    <row r="443"/>
+    <row r="444"/>
+    <row r="445"/>
+    <row r="446"/>
+    <row r="447"/>
+    <row r="448"/>
+    <row r="449"/>
+    <row r="450"/>
+    <row r="451"/>
+    <row r="452"/>
+    <row r="453"/>
+    <row r="454"/>
+    <row r="455"/>
+    <row r="456"/>
+    <row r="457"/>
+    <row r="458"/>
+    <row r="459"/>
+    <row r="460"/>
+    <row r="461"/>
+    <row r="462"/>
+    <row r="463"/>
+    <row r="464"/>
+    <row r="465"/>
+    <row r="466"/>
+    <row r="467"/>
+    <row r="468"/>
+    <row r="469"/>
+    <row r="470"/>
+    <row r="471"/>
+    <row r="472"/>
+    <row r="473"/>
+    <row r="474"/>
+    <row r="475"/>
+    <row r="476"/>
+    <row r="477"/>
+    <row r="478"/>
+    <row r="479"/>
+    <row r="480"/>
+    <row r="481"/>
+    <row r="482"/>
+    <row r="483"/>
+    <row r="484"/>
+    <row r="485"/>
+    <row r="486"/>
+    <row r="487"/>
+    <row r="488"/>
+    <row r="489"/>
+    <row r="490"/>
+    <row r="491"/>
+    <row r="492"/>
+    <row r="493"/>
+    <row r="494"/>
+    <row r="495"/>
+    <row r="496"/>
+    <row r="497"/>
+    <row r="498"/>
+    <row r="499"/>
+    <row r="500"/>
+    <row r="501"/>
+    <row r="502"/>
+    <row r="503"/>
+    <row r="504"/>
+    <row r="505"/>
+    <row r="506"/>
+    <row r="507"/>
+    <row r="508"/>
+    <row r="509"/>
+    <row r="510"/>
+    <row r="511"/>
+    <row r="512"/>
+    <row r="513"/>
+    <row r="514"/>
+    <row r="515"/>
+    <row r="516"/>
+    <row r="517"/>
+    <row r="518"/>
+    <row r="519"/>
+    <row r="520"/>
+    <row r="521"/>
+    <row r="522"/>
+    <row r="523"/>
+    <row r="524"/>
+    <row r="525"/>
+    <row r="526"/>
+    <row r="527"/>
+    <row r="528"/>
+    <row r="529"/>
+    <row r="530"/>
+    <row r="531"/>
+    <row r="532"/>
+    <row r="533"/>
+    <row r="534"/>
+    <row r="535"/>
+    <row r="536"/>
+    <row r="537"/>
+    <row r="538"/>
+    <row r="539"/>
+    <row r="540"/>
+    <row r="541"/>
+    <row r="542"/>
+    <row r="543"/>
+    <row r="544"/>
+    <row r="545"/>
+    <row r="546"/>
+    <row r="547"/>
+    <row r="548"/>
+    <row r="549"/>
+    <row r="550"/>
+    <row r="551"/>
+    <row r="552"/>
+    <row r="553"/>
+    <row r="554"/>
+    <row r="555"/>
+    <row r="556"/>
+    <row r="557"/>
+    <row r="558"/>
+    <row r="559"/>
+    <row r="560"/>
+    <row r="561"/>
+    <row r="562"/>
+    <row r="563"/>
+    <row r="564"/>
+    <row r="565"/>
+    <row r="566"/>
+    <row r="567"/>
+    <row r="568"/>
+    <row r="569"/>
+    <row r="570"/>
+    <row r="571"/>
+    <row r="572"/>
+    <row r="573"/>
+    <row r="574"/>
+    <row r="575"/>
+    <row r="576"/>
+    <row r="577"/>
+    <row r="578"/>
+    <row r="579"/>
+    <row r="580"/>
+    <row r="581"/>
+    <row r="582"/>
+    <row r="583"/>
+    <row r="584"/>
+    <row r="585"/>
+    <row r="586"/>
+    <row r="587"/>
+    <row r="588"/>
+    <row r="589"/>
+    <row r="590"/>
+    <row r="591"/>
+    <row r="592"/>
+    <row r="593"/>
+    <row r="594"/>
+    <row r="595"/>
+    <row r="596"/>
+    <row r="597"/>
+    <row r="598"/>
+    <row r="599"/>
+    <row r="600"/>
+    <row r="601"/>
+    <row r="602"/>
+    <row r="603"/>
+    <row r="604"/>
+    <row r="605"/>
+    <row r="606"/>
+    <row r="607"/>
+    <row r="608"/>
+    <row r="609"/>
+    <row r="610"/>
+    <row r="611"/>
+    <row r="612"/>
+    <row r="613"/>
+    <row r="614"/>
+    <row r="615"/>
+    <row r="616"/>
+    <row r="617"/>
+    <row r="618"/>
+    <row r="619"/>
+    <row r="620"/>
+    <row r="621"/>
+    <row r="622"/>
+    <row r="623"/>
+    <row r="624"/>
+    <row r="625"/>
+    <row r="626"/>
+    <row r="627"/>
+    <row r="628"/>
+    <row r="629"/>
+    <row r="630"/>
+    <row r="631"/>
+    <row r="632"/>
+    <row r="633"/>
+    <row r="634"/>
+    <row r="635"/>
+    <row r="636"/>
+    <row r="637"/>
+    <row r="638"/>
+    <row r="639"/>
+    <row r="640"/>
+    <row r="641"/>
+    <row r="642"/>
+    <row r="643"/>
+    <row r="644"/>
+    <row r="645"/>
+    <row r="646"/>
+    <row r="647"/>
+    <row r="648"/>
+    <row r="649"/>
+    <row r="650"/>
+    <row r="651"/>
+    <row r="652"/>
+    <row r="653"/>
+    <row r="654"/>
+    <row r="655"/>
+    <row r="656"/>
+    <row r="657"/>
+    <row r="658"/>
+    <row r="659"/>
+    <row r="660"/>
+    <row r="661"/>
+    <row r="662"/>
+    <row r="663"/>
+    <row r="664"/>
+    <row r="665"/>
+    <row r="666"/>
+    <row r="667"/>
+    <row r="668"/>
+    <row r="669"/>
+    <row r="670"/>
+    <row r="671"/>
+    <row r="672"/>
+    <row r="673"/>
+    <row r="674"/>
+    <row r="675"/>
+    <row r="676"/>
+    <row r="677"/>
+    <row r="678"/>
+    <row r="679"/>
+    <row r="680"/>
+    <row r="681"/>
+    <row r="682"/>
+    <row r="683"/>
+    <row r="684"/>
+    <row r="685"/>
+    <row r="686"/>
+    <row r="687"/>
+    <row r="688"/>
+    <row r="689"/>
+    <row r="690"/>
+    <row r="691"/>
+    <row r="692"/>
+    <row r="693"/>
+    <row r="694"/>
+    <row r="695"/>
+    <row r="696"/>
+    <row r="697"/>
+    <row r="698"/>
+    <row r="699"/>
+    <row r="700"/>
+    <row r="701"/>
+    <row r="702"/>
+    <row r="703"/>
+    <row r="704"/>
+    <row r="705"/>
+    <row r="706"/>
+    <row r="707"/>
+    <row r="708"/>
+    <row r="709"/>
+    <row r="710"/>
+    <row r="711"/>
+    <row r="712"/>
+    <row r="713"/>
+    <row r="714"/>
+    <row r="715"/>
+    <row r="716"/>
+    <row r="717"/>
+    <row r="718"/>
+    <row r="719"/>
+    <row r="720"/>
+    <row r="721"/>
+    <row r="722"/>
+    <row r="723"/>
+    <row r="724"/>
+    <row r="725"/>
+    <row r="726"/>
+    <row r="727"/>
+    <row r="728"/>
+    <row r="729"/>
+    <row r="730"/>
+    <row r="731"/>
+    <row r="732"/>
+    <row r="733"/>
+    <row r="734"/>
+    <row r="735"/>
+    <row r="736"/>
+    <row r="737"/>
+    <row r="738"/>
+    <row r="739"/>
+    <row r="740"/>
+    <row r="741"/>
+    <row r="742"/>
+    <row r="743"/>
+    <row r="744"/>
+    <row r="745"/>
+    <row r="746"/>
+    <row r="747"/>
+    <row r="748"/>
+    <row r="749"/>
+    <row r="750"/>
+    <row r="751"/>
+    <row r="752"/>
+    <row r="753"/>
+    <row r="754"/>
+    <row r="755"/>
+    <row r="756"/>
+    <row r="757"/>
+    <row r="758"/>
+    <row r="759"/>
+    <row r="760"/>
+    <row r="761"/>
+    <row r="762"/>
+    <row r="763"/>
+    <row r="764"/>
+    <row r="765"/>
+    <row r="766"/>
+    <row r="767"/>
+    <row r="768"/>
+    <row r="769"/>
+    <row r="770"/>
+    <row r="771"/>
+    <row r="772"/>
+    <row r="773"/>
+    <row r="774"/>
+    <row r="775"/>
+    <row r="776"/>
+    <row r="777"/>
+    <row r="778"/>
+    <row r="779"/>
+    <row r="780"/>
+    <row r="781"/>
+    <row r="782"/>
+    <row r="783"/>
+    <row r="784"/>
+    <row r="785"/>
+    <row r="786"/>
+    <row r="787"/>
+    <row r="788"/>
+    <row r="789"/>
+    <row r="790"/>
+    <row r="791"/>
+    <row r="792"/>
+    <row r="793"/>
+    <row r="794"/>
+    <row r="795"/>
+    <row r="796"/>
+    <row r="797"/>
+    <row r="798"/>
+    <row r="799"/>
+    <row r="800"/>
+    <row r="801"/>
+    <row r="802"/>
+    <row r="803"/>
+    <row r="804"/>
+    <row r="805"/>
+    <row r="806"/>
+    <row r="807"/>
+    <row r="808"/>
+    <row r="809"/>
+    <row r="810"/>
+    <row r="811"/>
+    <row r="812"/>
+    <row r="813"/>
+    <row r="814"/>
+    <row r="815"/>
+    <row r="816"/>
+    <row r="817"/>
+    <row r="818"/>
+    <row r="819"/>
+    <row r="820"/>
+    <row r="821"/>
+    <row r="822"/>
+    <row r="823"/>
+    <row r="824"/>
+    <row r="825"/>
+    <row r="826"/>
+    <row r="827"/>
+    <row r="828"/>
+    <row r="829"/>
+    <row r="830"/>
+    <row r="831"/>
+    <row r="832"/>
+    <row r="833"/>
+    <row r="834"/>
+    <row r="835"/>
+    <row r="836"/>
+    <row r="837"/>
+    <row r="838"/>
+    <row r="839"/>
+    <row r="840"/>
+    <row r="841"/>
+    <row r="842"/>
+    <row r="843"/>
+    <row r="844"/>
+    <row r="845"/>
+    <row r="846"/>
+    <row r="847"/>
+    <row r="848"/>
+    <row r="849"/>
+    <row r="850"/>
+    <row r="851"/>
+    <row r="852"/>
+    <row r="853"/>
+    <row r="854"/>
+    <row r="855"/>
+    <row r="856"/>
+    <row r="857"/>
+    <row r="858"/>
+    <row r="859"/>
+    <row r="860"/>
+    <row r="861"/>
+    <row r="862"/>
+    <row r="863"/>
+    <row r="864"/>
+    <row r="865"/>
+    <row r="866"/>
+    <row r="867"/>
+    <row r="868"/>
+    <row r="869"/>
+    <row r="870"/>
+    <row r="871"/>
+    <row r="872"/>
+    <row r="873"/>
+    <row r="874"/>
+    <row r="875"/>
+    <row r="876"/>
+    <row r="877"/>
+    <row r="878"/>
+    <row r="879"/>
+    <row r="880"/>
+    <row r="881"/>
+    <row r="882"/>
+    <row r="883"/>
+    <row r="884"/>
+    <row r="885"/>
+    <row r="886"/>
+    <row r="887"/>
+    <row r="888"/>
+    <row r="889"/>
+    <row r="890"/>
+    <row r="891"/>
+    <row r="892"/>
+    <row r="893"/>
+    <row r="894"/>
+    <row r="895"/>
+    <row r="896"/>
+    <row r="897"/>
+    <row r="898"/>
+    <row r="899"/>
+    <row r="900"/>
+    <row r="901"/>
+    <row r="902"/>
+    <row r="903"/>
+    <row r="904"/>
+    <row r="905"/>
+    <row r="906"/>
+    <row r="907"/>
+    <row r="908"/>
+    <row r="909"/>
+    <row r="910"/>
+    <row r="911"/>
+    <row r="912"/>
+    <row r="913"/>
+    <row r="914"/>
+    <row r="915"/>
+    <row r="916"/>
+    <row r="917"/>
+    <row r="918"/>
+    <row r="919"/>
+    <row r="920"/>
+    <row r="921"/>
+    <row r="922"/>
+    <row r="923"/>
+    <row r="924"/>
+    <row r="925"/>
+    <row r="926"/>
+    <row r="927"/>
+    <row r="928"/>
+    <row r="929"/>
+    <row r="930"/>
+    <row r="931"/>
+    <row r="932"/>
+    <row r="933"/>
+    <row r="934"/>
+    <row r="935"/>
+    <row r="936"/>
+    <row r="937"/>
+    <row r="938"/>
+    <row r="939"/>
+    <row r="940"/>
+    <row r="941"/>
+    <row r="942"/>
+    <row r="943"/>
+    <row r="944"/>
+    <row r="945"/>
+    <row r="946"/>
+    <row r="947"/>
+    <row r="948"/>
+    <row r="949"/>
+    <row r="950"/>
+    <row r="951"/>
+    <row r="952"/>
+    <row r="953"/>
+    <row r="954"/>
+    <row r="955"/>
+    <row r="956"/>
+    <row r="957"/>
+    <row r="958"/>
+    <row r="959"/>
+    <row r="960"/>
+    <row r="961"/>
+    <row r="962"/>
+    <row r="963"/>
+    <row r="964"/>
+    <row r="965"/>
+    <row r="966"/>
+    <row r="967"/>
+    <row r="968"/>
+    <row r="969"/>
+    <row r="970"/>
+    <row r="971"/>
+    <row r="972"/>
+    <row r="973"/>
+    <row r="974"/>
+    <row r="975"/>
+    <row r="976"/>
+    <row r="977"/>
+    <row r="978"/>
+    <row r="979"/>
+    <row r="980"/>
+    <row r="981"/>
+    <row r="982"/>
+    <row r="983"/>
+    <row r="984"/>
+    <row r="985"/>
+    <row r="986"/>
+    <row r="987"/>
+    <row r="988"/>
+    <row r="989"/>
+    <row r="990"/>
+    <row r="991"/>
+    <row r="992"/>
+    <row r="993"/>
+    <row r="994"/>
+    <row r="995"/>
+    <row r="996"/>
+    <row r="997"/>
+    <row r="998"/>
+    <row r="999"/>
+    <row r="1000"/>
+    <row r="1001"/>
+    <row r="1002"/>
+    <row r="1003"/>
+    <row r="1004"/>
+    <row r="1005"/>
+    <row r="1006"/>
+    <row r="1007"/>
+    <row r="1008"/>
+    <row r="1009"/>
+    <row r="1010"/>
+    <row r="1011"/>
+    <row r="1012"/>
+    <row r="1013"/>
+    <row r="1014"/>
+    <row r="1015"/>
+    <row r="1016"/>
+    <row r="1017"/>
+    <row r="1018"/>
+    <row r="1019"/>
+    <row r="1020"/>
+    <row r="1021"/>
+    <row r="1022"/>
+    <row r="1023"/>
+    <row r="1024"/>
+    <row r="1025"/>
+    <row r="1026"/>
+    <row r="1027"/>
+    <row r="1028"/>
+    <row r="1029"/>
+    <row r="1030"/>
+    <row r="1031"/>
+    <row r="1032"/>
+    <row r="1033"/>
+    <row r="1034"/>
+    <row r="1035"/>
+    <row r="1036"/>
+    <row r="1037"/>
+    <row r="1038"/>
+    <row r="1039"/>
+    <row r="1040"/>
+    <row r="1041"/>
+    <row r="1042"/>
+    <row r="1043"/>
+    <row r="1044"/>
+    <row r="1045"/>
+    <row r="1046"/>
+    <row r="1047"/>
+    <row r="1048"/>
+    <row r="1049"/>
+    <row r="1050"/>
+    <row r="1051"/>
+    <row r="1052"/>
+    <row r="1053"/>
+    <row r="1054"/>
+    <row r="1055"/>
+    <row r="1056"/>
+    <row r="1057"/>
+    <row r="1058"/>
+    <row r="1059"/>
+    <row r="1060"/>
+    <row r="1061"/>
+    <row r="1062"/>
+    <row r="1063"/>
+    <row r="1064"/>
+    <row r="1065"/>
+    <row r="1066"/>
+    <row r="1067"/>
+    <row r="1068"/>
+    <row r="1069"/>
+    <row r="1070"/>
+    <row r="1071"/>
+    <row r="1072"/>
+    <row r="1073"/>
+    <row r="1074"/>
+    <row r="1075"/>
+    <row r="1076"/>
+    <row r="1077"/>
+    <row r="1078"/>
+    <row r="1079"/>
+    <row r="1080"/>
+    <row r="1081"/>
+    <row r="1082"/>
+    <row r="1083"/>
+    <row r="1084"/>
+    <row r="1085"/>
+    <row r="1086"/>
+    <row r="1087"/>
+    <row r="1088"/>
+    <row r="1089"/>
+    <row r="1090"/>
+    <row r="1091"/>
+    <row r="1092"/>
+    <row r="1093"/>
+    <row r="1094"/>
+    <row r="1095"/>
+    <row r="1096"/>
+    <row r="1097"/>
+    <row r="1098"/>
+    <row r="1099"/>
+    <row r="1100"/>
+    <row r="1101"/>
+    <row r="1102"/>
+    <row r="1103"/>
+    <row r="1104"/>
+    <row r="1105"/>
+    <row r="1106"/>
+    <row r="1107"/>
+    <row r="1108"/>
+    <row r="1109"/>
+    <row r="1110"/>
+    <row r="1111"/>
+    <row r="1112"/>
+    <row r="1113"/>
+    <row r="1114"/>
+    <row r="1115"/>
+    <row r="1116"/>
+    <row r="1117"/>
+    <row r="1118"/>
+    <row r="1119"/>
+    <row r="1120"/>
+    <row r="1121"/>
+    <row r="1122"/>
+    <row r="1123"/>
+    <row r="1124"/>
+    <row r="1125"/>
+    <row r="1126"/>
+    <row r="1127"/>
+    <row r="1128"/>
+    <row r="1129"/>
+    <row r="1130"/>
+    <row r="1131"/>
+    <row r="1132"/>
+    <row r="1133"/>
+    <row r="1134"/>
+    <row r="1135"/>
+    <row r="1136"/>
+    <row r="1137"/>
+    <row r="1138"/>
+    <row r="1139"/>
+    <row r="1140"/>
+    <row r="1141"/>
+    <row r="1142"/>
+    <row r="1143"/>
+    <row r="1144"/>
+    <row r="1145"/>
+    <row r="1146"/>
+    <row r="1147"/>
+    <row r="1148"/>
+    <row r="1149"/>
+    <row r="1150"/>
+    <row r="1151"/>
+    <row r="1152"/>
+    <row r="1153"/>
+    <row r="1154"/>
+    <row r="1155"/>
+    <row r="1156"/>
+    <row r="1157"/>
+    <row r="1158"/>
+    <row r="1159"/>
+    <row r="1160"/>
+    <row r="1161"/>
+    <row r="1162"/>
+    <row r="1163"/>
+    <row r="1164"/>
+    <row r="1165"/>
+    <row r="1166"/>
+    <row r="1167"/>
+    <row r="1168"/>
+    <row r="1169"/>
+    <row r="1170"/>
+    <row r="1171"/>
+    <row r="1172"/>
+    <row r="1173"/>
+    <row r="1174"/>
+    <row r="1175"/>
+    <row r="1176"/>
+    <row r="1177"/>
+    <row r="1178"/>
+    <row r="1179"/>
+    <row r="1180"/>
+    <row r="1181"/>
+    <row r="1182"/>
+    <row r="1183"/>
+    <row r="1184"/>
+    <row r="1185"/>
+    <row r="1186"/>
+    <row r="1187"/>
+    <row r="1188"/>
+    <row r="1189"/>
+    <row r="1190"/>
+    <row r="1191"/>
+    <row r="1192"/>
+    <row r="1193"/>
+    <row r="1194"/>
+    <row r="1195"/>
+    <row r="1196"/>
+    <row r="1197"/>
+    <row r="1198"/>
+    <row r="1199"/>
+    <row r="1200"/>
+    <row r="1201"/>
+    <row r="1202"/>
+    <row r="1203"/>
+    <row r="1204"/>
+    <row r="1205"/>
+    <row r="1206"/>
+    <row r="1207"/>
+    <row r="1208"/>
+    <row r="1209"/>
+    <row r="1210"/>
+    <row r="1211"/>
+    <row r="1212"/>
+    <row r="1213"/>
+    <row r="1214"/>
+    <row r="1215"/>
+    <row r="1216"/>
+    <row r="1217"/>
+    <row r="1218"/>
+    <row r="1219"/>
+    <row r="1220"/>
+    <row r="1221"/>
+    <row r="1222"/>
+    <row r="1223"/>
+    <row r="1224"/>
+    <row r="1225"/>
+    <row r="1226"/>
+    <row r="1227"/>
+    <row r="1228"/>
+    <row r="1229"/>
+    <row r="1230"/>
+    <row r="1231"/>
+    <row r="1232"/>
+    <row r="1233"/>
+    <row r="1234"/>
+    <row r="1235"/>
+    <row r="1236"/>
+    <row r="1237"/>
+    <row r="1238"/>
+    <row r="1239"/>
+    <row r="1240"/>
+    <row r="1241"/>
+    <row r="1242"/>
+    <row r="1243"/>
+    <row r="1244"/>
+    <row r="1245"/>
+    <row r="1246"/>
+    <row r="1247"/>
+    <row r="1248"/>
+    <row r="1249"/>
+    <row r="1250"/>
+    <row r="1251"/>
+    <row r="1252"/>
+    <row r="1253"/>
+    <row r="1254"/>
+    <row r="1255"/>
+    <row r="1256"/>
+    <row r="1257"/>
+    <row r="1258"/>
+    <row r="1259"/>
+    <row r="1260"/>
+    <row r="1261"/>
+    <row r="1262"/>
+    <row r="1263"/>
+    <row r="1264"/>
+    <row r="1265"/>
+    <row r="1266"/>
+    <row r="1267"/>
+    <row r="1268"/>
+    <row r="1269"/>
+    <row r="1270"/>
+    <row r="1271"/>
+    <row r="1272"/>
+    <row r="1273"/>
+    <row r="1274"/>
+    <row r="1275"/>
+    <row r="1276"/>
+    <row r="1277"/>
+    <row r="1278"/>
+    <row r="1279"/>
+    <row r="1280"/>
+    <row r="1281"/>
+    <row r="1282"/>
+    <row r="1283"/>
+    <row r="1284"/>
+    <row r="1285"/>
+    <row r="1286"/>
+    <row r="1287"/>
+    <row r="1288"/>
+    <row r="1289"/>
+    <row r="1290"/>
+    <row r="1291"/>
+    <row r="1292"/>
+    <row r="1293"/>
+    <row r="1294"/>
+    <row r="1295"/>
+    <row r="1296"/>
+    <row r="1297"/>
+    <row r="1298"/>
+    <row r="1299"/>
+    <row r="1300"/>
+    <row r="1301"/>
+    <row r="1302"/>
+    <row r="1303"/>
+    <row r="1304"/>
+    <row r="1305"/>
+    <row r="1306"/>
+    <row r="1307"/>
+    <row r="1308"/>
+    <row r="1309"/>
+    <row r="1310"/>
+    <row r="1311"/>
+    <row r="1312"/>
+    <row r="1313"/>
+    <row r="1314"/>
+    <row r="1315"/>
+    <row r="1316"/>
+    <row r="1317"/>
+    <row r="1318"/>
+    <row r="1319"/>
+    <row r="1320"/>
+    <row r="1321"/>
+    <row r="1322"/>
+    <row r="1323"/>
+    <row r="1324"/>
+    <row r="1325"/>
+    <row r="1326"/>
+    <row r="1327"/>
+    <row r="1328"/>
+    <row r="1329"/>
+    <row r="1330"/>
+    <row r="1331"/>
+    <row r="1332"/>
+    <row r="1333"/>
+    <row r="1334"/>
+    <row r="1335"/>
+    <row r="1336"/>
+    <row r="1337"/>
+    <row r="1338"/>
+    <row r="1339"/>
+    <row r="1340"/>
+    <row r="1341"/>
+    <row r="1342"/>
+    <row r="1343"/>
+    <row r="1344"/>
+    <row r="1345"/>
+    <row r="1346"/>
+    <row r="1347"/>
+    <row r="1348"/>
+    <row r="1349"/>
+    <row r="1350"/>
+    <row r="1351"/>
+    <row r="1352"/>
+    <row r="1353"/>
+    <row r="1354"/>
+    <row r="1355"/>
+    <row r="1356"/>
+    <row r="1357"/>
+    <row r="1358"/>
+    <row r="1359"/>
+    <row r="1360"/>
+    <row r="1361"/>
+    <row r="1362"/>
+    <row r="1363"/>
+    <row r="1364"/>
+    <row r="1365"/>
+    <row r="1366"/>
+    <row r="1367"/>
+    <row r="1368"/>
+    <row r="1369"/>
+    <row r="1370"/>
+    <row r="1371"/>
+    <row r="1372"/>
+    <row r="1373"/>
+    <row r="1374"/>
+    <row r="1375"/>
+    <row r="1376"/>
+    <row r="1377"/>
+    <row r="1378"/>
+    <row r="1379"/>
+    <row r="1380"/>
+    <row r="1381"/>
+    <row r="1382"/>
+    <row r="1383"/>
+    <row r="1384"/>
+    <row r="1385"/>
+    <row r="1386"/>
+    <row r="1387"/>
+    <row r="1388"/>
+    <row r="1389"/>
+    <row r="1390"/>
+    <row r="1391"/>
+    <row r="1392"/>
+    <row r="1393"/>
+    <row r="1394"/>
+    <row r="1395"/>
+    <row r="1396"/>
+    <row r="1397"/>
+    <row r="1398"/>
+    <row r="1399"/>
+    <row r="1400"/>
+    <row r="1401"/>
+    <row r="1402"/>
+    <row r="1403"/>
+    <row r="1404"/>
+    <row r="1405"/>
+    <row r="1406"/>
+    <row r="1407"/>
+    <row r="1408"/>
+    <row r="1409"/>
+    <row r="1410"/>
+    <row r="1411"/>
+    <row r="1412"/>
+    <row r="1413"/>
+    <row r="1414"/>
+    <row r="1415"/>
+    <row r="1416"/>
+    <row r="1417"/>
+    <row r="1418"/>
+    <row r="1419"/>
+    <row r="1420"/>
+    <row r="1421"/>
+    <row r="1422"/>
+    <row r="1423"/>
+    <row r="1424"/>
+    <row r="1425"/>
+    <row r="1426"/>
+    <row r="1427"/>
+    <row r="1428"/>
+    <row r="1429"/>
+    <row r="1430"/>
+    <row r="1431"/>
+    <row r="1432"/>
+    <row r="1433"/>
+    <row r="1434"/>
+    <row r="1435"/>
+    <row r="1436"/>
+    <row r="1437"/>
+    <row r="1438"/>
+    <row r="1439"/>
+    <row r="1440"/>
+    <row r="1441"/>
+    <row r="1442"/>
+    <row r="1443"/>
+    <row r="1444"/>
+    <row r="1445"/>
+    <row r="1446"/>
+    <row r="1447"/>
+    <row r="1448"/>
+    <row r="1449"/>
+    <row r="1450"/>
+    <row r="1451"/>
+    <row r="1452"/>
+    <row r="1453"/>
+    <row r="1454"/>
+    <row r="1455"/>
+    <row r="1456"/>
+    <row r="1457"/>
+    <row r="1458"/>
+    <row r="1459"/>
+    <row r="1460"/>
+    <row r="1461"/>
+    <row r="1462"/>
+    <row r="1463"/>
+    <row r="1464"/>
+    <row r="1465"/>
+    <row r="1466"/>
+    <row r="1467"/>
+    <row r="1468"/>
+    <row r="1469"/>
+    <row r="1470"/>
+    <row r="1471"/>
+    <row r="1472"/>
+    <row r="1473"/>
+    <row r="1474"/>
+    <row r="1475"/>
+    <row r="1476"/>
+    <row r="1477"/>
+    <row r="1478"/>
+    <row r="1479"/>
+    <row r="1480"/>
+    <row r="1481"/>
+    <row r="1482"/>
+    <row r="1483"/>
+    <row r="1484"/>
+    <row r="1485"/>
+    <row r="1486"/>
+    <row r="1487"/>
+    <row r="1488"/>
+    <row r="1489"/>
+    <row r="1490"/>
+    <row r="1491"/>
+    <row r="1492"/>
+    <row r="1493"/>
+    <row r="1494"/>
+    <row r="1495"/>
+    <row r="1496"/>
+    <row r="1497"/>
+    <row r="1498"/>
+    <row r="1499"/>
+    <row r="1500"/>
+    <row r="1501"/>
+    <row r="1502"/>
+    <row r="1503"/>
+    <row r="1504"/>
+    <row r="1505"/>
+    <row r="1506"/>
+    <row r="1507"/>
+    <row r="1508"/>
+    <row r="1509"/>
+    <row r="1510"/>
+    <row r="1511"/>
+    <row r="1512"/>
+    <row r="1513"/>
+    <row r="1514"/>
+    <row r="1515"/>
+    <row r="1516"/>
+    <row r="1517"/>
+    <row r="1518"/>
+    <row r="1519"/>
+    <row r="1520"/>
+    <row r="1521"/>
+    <row r="1522"/>
+    <row r="1523"/>
+    <row r="1524"/>
+    <row r="1525"/>
+    <row r="1526"/>
+    <row r="1527"/>
+    <row r="1528"/>
+    <row r="1529"/>
+    <row r="1530"/>
+    <row r="1531"/>
+    <row r="1532"/>
+    <row r="1533"/>
+    <row r="1534"/>
+    <row r="1535"/>
+    <row r="1536"/>
+    <row r="1537"/>
+    <row r="1538"/>
+    <row r="1539"/>
+    <row r="1540"/>
+    <row r="1541"/>
+    <row r="1542"/>
+    <row r="1543"/>
+    <row r="1544"/>
+    <row r="1545"/>
+    <row r="1546"/>
+    <row r="1547"/>
+    <row r="1548"/>
+    <row r="1549"/>
+    <row r="1550"/>
+    <row r="1551"/>
+    <row r="1552"/>
+    <row r="1553"/>
+    <row r="1554"/>
+    <row r="1555"/>
+    <row r="1556"/>
+    <row r="1557"/>
+    <row r="1558"/>
+    <row r="1559"/>
+    <row r="1560"/>
+    <row r="1561"/>
+    <row r="1562"/>
+    <row r="1563"/>
+    <row r="1564"/>
+    <row r="1565"/>
+    <row r="1566"/>
+    <row r="1567"/>
+    <row r="1568"/>
+    <row r="1569"/>
+    <row r="1570"/>
+    <row r="1571"/>
+    <row r="1572"/>
+    <row r="1573"/>
+    <row r="1574"/>
+    <row r="1575"/>
+    <row r="1576"/>
+    <row r="1577"/>
+    <row r="1578"/>
+    <row r="1579"/>
+    <row r="1580"/>
+    <row r="1581"/>
+    <row r="1582"/>
+    <row r="1583"/>
+    <row r="1584"/>
+    <row r="1585"/>
+    <row r="1586"/>
+    <row r="1587"/>
+    <row r="1588"/>
+    <row r="1589"/>
+    <row r="1590"/>
+    <row r="1591"/>
+    <row r="1592"/>
+    <row r="1593"/>
+    <row r="1594"/>
+    <row r="1595"/>
+    <row r="1596"/>
+    <row r="1597"/>
+    <row r="1598"/>
+    <row r="1599"/>
+    <row r="1600"/>
+    <row r="1601"/>
+    <row r="1602"/>
+    <row r="1603"/>
+    <row r="1604"/>
+    <row r="1605"/>
+    <row r="1606"/>
+    <row r="1607"/>
+    <row r="1608"/>
+    <row r="1609"/>
+    <row r="1610"/>
+    <row r="1611"/>
+    <row r="1612"/>
+    <row r="1613"/>
+    <row r="1614"/>
+    <row r="1615"/>
+    <row r="1616"/>
+    <row r="1617"/>
+    <row r="1618"/>
+    <row r="1619"/>
+    <row r="1620"/>
+    <row r="1621"/>
+    <row r="1622"/>
+    <row r="1623"/>
+    <row r="1624"/>
+    <row r="1625"/>
+    <row r="1626"/>
+    <row r="1627"/>
+    <row r="1628"/>
+    <row r="1629"/>
+    <row r="1630"/>
+    <row r="1631"/>
+    <row r="1632"/>
+    <row r="1633"/>
+    <row r="1634"/>
+    <row r="1635"/>
+    <row r="1636"/>
+    <row r="1637"/>
+    <row r="1638"/>
+    <row r="1639"/>
+    <row r="1640"/>
+    <row r="1641"/>
+    <row r="1642"/>
+    <row r="1643"/>
+    <row r="1644"/>
+    <row r="1645"/>
+    <row r="1646"/>
+    <row r="1647"/>
+    <row r="1648"/>
+    <row r="1649"/>
+    <row r="1650"/>
+    <row r="1651"/>
+    <row r="1652"/>
+    <row r="1653"/>
+    <row r="1654"/>
+    <row r="1655"/>
+    <row r="1656"/>
+    <row r="1657"/>
+    <row r="1658"/>
+    <row r="1659"/>
+    <row r="1660"/>
+    <row r="1661"/>
+    <row r="1662"/>
+    <row r="1663"/>
+    <row r="1664"/>
+    <row r="1665"/>
+    <row r="1666"/>
+    <row r="1667"/>
+    <row r="1668"/>
+    <row r="1669"/>
+    <row r="1670"/>
+    <row r="1671"/>
+    <row r="1672"/>
+    <row r="1673"/>
+    <row r="1674"/>
+    <row r="1675"/>
+    <row r="1676"/>
+    <row r="1677"/>
+    <row r="1678"/>
+    <row r="1679"/>
+    <row r="1680"/>
+    <row r="1681"/>
+    <row r="1682"/>
+    <row r="1683"/>
+    <row r="1684"/>
+    <row r="1685"/>
+    <row r="1686"/>
+    <row r="1687"/>
+    <row r="1688"/>
+    <row r="1689"/>
+    <row r="1690"/>
+    <row r="1691"/>
+    <row r="1692"/>
+    <row r="1693"/>
+    <row r="1694"/>
+    <row r="1695"/>
+    <row r="1696"/>
+    <row r="1697"/>
+    <row r="1698"/>
+    <row r="1699"/>
+    <row r="1700"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:B1"/>
@@ -16546,10 +18014,10 @@
   <dimension ref="B2:E110"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.89453125" defaultRowHeight="12.75" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="19.77" customWidth="1" style="42" min="2" max="2"/>
-    <col width="19.78" customWidth="1" style="42" min="3" max="3"/>
-    <col width="17.16" customWidth="1" style="42" min="4" max="4"/>
-    <col width="29.63" customWidth="1" style="42" min="5" max="5"/>
+    <col width="19.77" customWidth="1" style="75" min="2" max="2"/>
+    <col width="19.78" customWidth="1" style="75" min="3" max="3"/>
+    <col width="17.16" customWidth="1" style="75" min="4" max="4"/>
+    <col width="29.63" customWidth="1" style="75" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="2" ht="12.75" customHeight="1" s="69">
@@ -16582,7 +18050,7 @@
         </is>
       </c>
       <c r="D3" s="77" t="n"/>
-      <c r="E3" s="42" t="inlineStr">
+      <c r="E3" s="75" t="inlineStr">
         <is>
           <t>2XS</t>
         </is>
@@ -17381,8 +18849,8 @@
   <dimension ref="A1:B60"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.48828125" defaultRowHeight="12.75" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="54.83" customWidth="1" style="42" min="1" max="1"/>
-    <col width="215.56" customWidth="1" style="42" min="2" max="2"/>
+    <col width="54.83" customWidth="1" style="75" min="1" max="1"/>
+    <col width="215.56" customWidth="1" style="75" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="69">
@@ -17398,7 +18866,7 @@
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="69">
-      <c r="A2" s="80" t="inlineStr">
+      <c r="A2" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000001&gt; АРАФАТКА</t>
         </is>
@@ -17410,7 +18878,7 @@
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="69">
-      <c r="A3" s="80" t="inlineStr">
+      <c r="A3" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000002&gt; БАБОЧКА</t>
         </is>
@@ -17422,7 +18890,7 @@
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="69">
-      <c r="A4" s="80" t="inlineStr">
+      <c r="A4" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000003&gt; БАЛАКЛАВА</t>
         </is>
@@ -17434,7 +18902,7 @@
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="69">
-      <c r="A5" s="80" t="inlineStr">
+      <c r="A5" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000004&gt; БАНДАНА</t>
         </is>
@@ -17446,7 +18914,7 @@
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="69">
-      <c r="A6" s="80" t="inlineStr">
+      <c r="A6" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000005&gt; БАНТ</t>
         </is>
@@ -17458,7 +18926,7 @@
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="69">
-      <c r="A7" s="80" t="inlineStr">
+      <c r="A7" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000006&gt; БАСКА</t>
         </is>
@@ -17470,7 +18938,7 @@
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="69">
-      <c r="A8" s="80" t="inlineStr">
+      <c r="A8" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000007&gt; БАФФ</t>
         </is>
@@ -17482,7 +18950,7 @@
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="69">
-      <c r="A9" s="80" t="inlineStr">
+      <c r="A9" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000008&gt; ВОРОТНИК</t>
         </is>
@@ -17506,7 +18974,7 @@
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="69">
-      <c r="A11" s="80" t="inlineStr">
+      <c r="A11" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000009&gt; ВУАЛЬ</t>
         </is>
@@ -17518,7 +18986,7 @@
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="69">
-      <c r="A12" s="80" t="inlineStr">
+      <c r="A12" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000010&gt; ГАЛСТУК</t>
         </is>
@@ -17530,7 +18998,7 @@
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="69">
-      <c r="A13" s="80" t="inlineStr">
+      <c r="A13" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000011&gt; ГАЛСТУК-БАБОЧКА</t>
         </is>
@@ -17542,7 +19010,7 @@
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="69">
-      <c r="A14" s="80" t="inlineStr">
+      <c r="A14" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000012&gt; ГЕЙТОР</t>
         </is>
@@ -17554,7 +19022,7 @@
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="69">
-      <c r="A15" s="80" t="inlineStr">
+      <c r="A15" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000013&gt; ГОРЖЕТКА</t>
         </is>
@@ -17574,7 +19042,7 @@
       <c r="B16" s="84" t="n"/>
     </row>
     <row r="17" ht="15" customHeight="1" s="69">
-      <c r="A17" s="80" t="inlineStr">
+      <c r="A17" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000014&gt; ДИАДЕМА</t>
         </is>
@@ -17582,7 +19050,7 @@
       <c r="B17" s="84" t="n"/>
     </row>
     <row r="18" ht="48.75" customHeight="1" s="69">
-      <c r="A18" s="80" t="inlineStr">
+      <c r="A18" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000015&gt; ЖАБО</t>
         </is>
@@ -17590,7 +19058,7 @@
       <c r="B18" s="84" t="n"/>
     </row>
     <row r="19" ht="30" customHeight="1" s="69">
-      <c r="A19" s="80" t="inlineStr">
+      <c r="A19" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000016&gt; ЗАКОЛКА</t>
         </is>
@@ -17598,7 +19066,7 @@
       <c r="B19" s="84" t="n"/>
     </row>
     <row r="20" ht="30" customHeight="1" s="69">
-      <c r="A20" s="80" t="inlineStr">
+      <c r="A20" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000017&gt; КАПЮШОН</t>
         </is>
@@ -17606,7 +19074,7 @@
       <c r="B20" s="84" t="n"/>
     </row>
     <row r="21" ht="30" customHeight="1" s="69">
-      <c r="A21" s="80" t="inlineStr">
+      <c r="A21" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000018&gt; КАШНЕ</t>
         </is>
@@ -17614,7 +19082,7 @@
       <c r="B21" s="84" t="n"/>
     </row>
     <row r="22" ht="15" customHeight="1" s="69">
-      <c r="A22" s="80" t="inlineStr">
+      <c r="A22" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000019&gt; КОСЫНКА</t>
         </is>
@@ -17622,7 +19090,7 @@
       <c r="B22" s="84" t="n"/>
     </row>
     <row r="23" ht="15" customHeight="1" s="69">
-      <c r="A23" s="80" t="inlineStr">
+      <c r="A23" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000020&gt; ЛЕНТА</t>
         </is>
@@ -17638,7 +19106,7 @@
       <c r="B24" s="84" t="n"/>
     </row>
     <row r="25" ht="15" customHeight="1" s="69">
-      <c r="A25" s="80" t="inlineStr">
+      <c r="A25" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000021&gt; МАНИШКА</t>
         </is>
@@ -17646,7 +19114,7 @@
       <c r="B25" s="84" t="n"/>
     </row>
     <row r="26" ht="34.5" customHeight="1" s="69">
-      <c r="A26" s="80" t="inlineStr">
+      <c r="A26" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000022&gt; МАНТИЛЬЯ</t>
         </is>
@@ -17654,7 +19122,7 @@
       <c r="B26" s="84" t="n"/>
     </row>
     <row r="27" ht="34.5" customHeight="1" s="69">
-      <c r="A27" s="80" t="inlineStr">
+      <c r="A27" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000023&gt; МАСКА</t>
         </is>
@@ -17662,7 +19130,7 @@
       <c r="B27" s="84" t="n"/>
     </row>
     <row r="28" ht="33" customHeight="1" s="69">
-      <c r="A28" s="80" t="inlineStr">
+      <c r="A28" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000024&gt; НАГРУДНИК</t>
         </is>
@@ -17670,7 +19138,7 @@
       <c r="B28" s="84" t="n"/>
     </row>
     <row r="29" ht="36" customHeight="1" s="69">
-      <c r="A29" s="80" t="inlineStr">
+      <c r="A29" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000025&gt; НАМАЗНИК</t>
         </is>
@@ -17686,7 +19154,7 @@
       <c r="B30" s="84" t="n"/>
     </row>
     <row r="31" ht="36.75" customHeight="1" s="69">
-      <c r="A31" s="80" t="inlineStr">
+      <c r="A31" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000026&gt; ПАЛАНТИН</t>
         </is>
@@ -17694,7 +19162,7 @@
       <c r="B31" s="84" t="n"/>
     </row>
     <row r="32" ht="25.5" customHeight="1" s="69">
-      <c r="A32" s="80" t="inlineStr">
+      <c r="A32" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000027&gt; ПАРЕО</t>
         </is>
@@ -17710,7 +19178,7 @@
       <c r="B33" s="84" t="n"/>
     </row>
     <row r="34" ht="39.75" customHeight="1" s="69">
-      <c r="A34" s="80" t="inlineStr">
+      <c r="A34" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000028&gt; ПЕЛЕНКА</t>
         </is>
@@ -17718,7 +19186,7 @@
       <c r="B34" s="84" t="n"/>
     </row>
     <row r="35" ht="15" customHeight="1" s="69">
-      <c r="A35" s="80" t="inlineStr">
+      <c r="A35" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000029&gt; ПЕЛЕРИНА</t>
         </is>
@@ -17726,7 +19194,7 @@
       <c r="B35" s="84" t="n"/>
     </row>
     <row r="36" ht="15" customHeight="1" s="69">
-      <c r="A36" s="80" t="inlineStr">
+      <c r="A36" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000030&gt; ПЛАТОК</t>
         </is>
@@ -17734,7 +19202,7 @@
       <c r="B36" s="84" t="n"/>
     </row>
     <row r="37" ht="15" customHeight="1" s="69">
-      <c r="A37" s="80" t="inlineStr">
+      <c r="A37" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000031&gt; ПЛАТОК ГОЛОВНОЙ</t>
         </is>
@@ -17742,7 +19210,7 @@
       <c r="B37" s="84" t="n"/>
     </row>
     <row r="38" ht="15" customHeight="1" s="69">
-      <c r="A38" s="80" t="inlineStr">
+      <c r="A38" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000032&gt; ПЛАТОК НОСОВОЙ</t>
         </is>
@@ -17750,7 +19218,7 @@
       <c r="B38" s="84" t="n"/>
     </row>
     <row r="39" ht="15" customHeight="1" s="69">
-      <c r="A39" s="80" t="inlineStr">
+      <c r="A39" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000033&gt; ПЛАТОК ШЕЙНЫЙ</t>
         </is>
@@ -17758,7 +19226,7 @@
       <c r="B39" s="84" t="n"/>
     </row>
     <row r="40" ht="15" customHeight="1" s="69">
-      <c r="A40" s="80" t="inlineStr">
+      <c r="A40" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000059&gt; ПОВЯЗКА НА ГОЛОВУ</t>
         </is>
@@ -17766,7 +19234,7 @@
       <c r="B40" s="84" t="n"/>
     </row>
     <row r="41" ht="15" customHeight="1" s="69">
-      <c r="A41" s="80" t="inlineStr">
+      <c r="A41" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000034&gt; ПОДТЯЖКИ</t>
         </is>
@@ -17774,7 +19242,7 @@
       <c r="B41" s="84" t="n"/>
     </row>
     <row r="42" ht="15" customHeight="1" s="69">
-      <c r="A42" s="80" t="inlineStr">
+      <c r="A42" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000035&gt; ПОДШЛЕМНИК</t>
         </is>
@@ -17782,7 +19250,7 @@
       <c r="B42" s="84" t="n"/>
     </row>
     <row r="43" ht="15" customHeight="1" s="69">
-      <c r="A43" s="80" t="inlineStr">
+      <c r="A43" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000036&gt; ПОРТУПЕЯ</t>
         </is>
@@ -17790,7 +19258,7 @@
       <c r="B43" s="84" t="n"/>
     </row>
     <row r="44" ht="15" customHeight="1" s="69">
-      <c r="A44" s="80" t="inlineStr">
+      <c r="A44" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000037&gt; ПОЯС</t>
         </is>
@@ -17798,7 +19266,7 @@
       <c r="B44" s="84" t="n"/>
     </row>
     <row r="45" ht="15" customHeight="1" s="69">
-      <c r="A45" s="80" t="inlineStr">
+      <c r="A45" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000038&gt; РЕЗИНКА НА ГОЛОВУ</t>
         </is>
@@ -17806,7 +19274,7 @@
       <c r="B45" s="84" t="n"/>
     </row>
     <row r="46" ht="13.5" customHeight="1" s="69">
-      <c r="A46" s="80" t="inlineStr">
+      <c r="A46" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000039&gt; РЕМЕНЬ</t>
         </is>
@@ -17814,7 +19282,7 @@
       <c r="B46" s="84" t="n"/>
     </row>
     <row r="47" ht="13.5" customHeight="1" s="69">
-      <c r="A47" s="80" t="inlineStr">
+      <c r="A47" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000052&gt; РУКАВА</t>
         </is>
@@ -17822,7 +19290,7 @@
       <c r="B47" s="84" t="n"/>
     </row>
     <row r="48" ht="15" customHeight="1" s="69">
-      <c r="A48" s="80" t="inlineStr">
+      <c r="A48" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000040&gt; СНУД</t>
         </is>
@@ -17830,7 +19298,7 @@
       <c r="B48" s="84" t="n"/>
     </row>
     <row r="49" ht="15" customHeight="1" s="69">
-      <c r="A49" s="80" t="inlineStr">
+      <c r="A49" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000041&gt; ТРЕССЫ</t>
         </is>
@@ -17838,7 +19306,7 @@
       <c r="B49" s="84" t="n"/>
     </row>
     <row r="50" ht="15" customHeight="1" s="69">
-      <c r="A50" s="80" t="inlineStr">
+      <c r="A50" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000042&gt; ФАТА</t>
         </is>
@@ -17846,7 +19314,7 @@
       <c r="B50" s="84" t="n"/>
     </row>
     <row r="51" ht="15" customHeight="1" s="69">
-      <c r="A51" s="80" t="inlineStr">
+      <c r="A51" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000043&gt; ХИДЖАБ</t>
         </is>
@@ -17854,7 +19322,7 @@
       <c r="B51" s="84" t="n"/>
     </row>
     <row r="52" ht="15" customHeight="1" s="69">
-      <c r="A52" s="80" t="inlineStr">
+      <c r="A52" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000044&gt; ХОМУТ</t>
         </is>
@@ -17862,7 +19330,7 @@
       <c r="B52" s="84" t="n"/>
     </row>
     <row r="53" ht="15" customHeight="1" s="69">
-      <c r="A53" s="80" t="inlineStr">
+      <c r="A53" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000045&gt; ЧАЛМА</t>
         </is>
@@ -17870,42 +19338,42 @@
       <c r="B53" s="84" t="n"/>
     </row>
     <row r="54" ht="15" customHeight="1" s="69">
-      <c r="A54" s="80" t="inlineStr">
+      <c r="A54" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000046&gt; ЧОКЕР</t>
         </is>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="69">
-      <c r="A55" s="80" t="inlineStr">
+      <c r="A55" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000047&gt; ШАЛЬ</t>
         </is>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="69">
-      <c r="A56" s="80" t="inlineStr">
+      <c r="A56" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000048&gt; ШАПКА-ШАРФ</t>
         </is>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="69">
-      <c r="A57" s="80" t="inlineStr">
+      <c r="A57" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000053&gt; ШАПОЧКА ДЛЯ ПЛАВАНИЯ</t>
         </is>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="69">
-      <c r="A58" s="80" t="inlineStr">
+      <c r="A58" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000049&gt; ШАРФ-СНУД</t>
         </is>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="69">
-      <c r="A59" s="80" t="inlineStr">
+      <c r="A59" s="85" t="inlineStr">
         <is>
           <t>&lt;4000000050&gt; ШАРФ-КАПЮШОН</t>
         </is>

</xml_diff>